<commit_message>
Resultados de la búsqueda 2026-10-16
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$K$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$K$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -498,12 +498,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tandazo — Autofinanciamiento $50k a $220k MXN sin intereses ni buró</t>
+          <t>PRO Network</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tandazo.com.mx/</t>
+          <t>https://www.pronetwork.mx/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -513,21 +513,21 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Mensualidad fija $2,500 MXN. Sin historial crediticio, sin aval. Comprueba solo capacidad de pago. 100% digital.</t>
+          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>contratos@tandazo.com.mx, privacidad@tandazo.com.mx</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>plataforma de inversión para mujeres México</t>
@@ -541,39 +541,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PRO Network</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.pronetwork.mx/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>usuario@dominio.com</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -584,12 +592,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://finantres.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -599,212 +607,208 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/visionarias.business/</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/finantres/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/visionarias</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>app para invertir para principiantes México</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/fintual/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>usuario@dominio.com</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Los 7 Mejores Brokers en Chile 2026 | Comparativa con Comisiones Reales</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.mejoresbrokers.cl/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Comparamos XTB, eToro, Fintual, Pepperstone e Interactive Brokers desde Chile. Comisiones reales, regulación CMF verificada, métodos de depósito locales. Actualizado abril 2026.</t>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>tu@email.com</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>app para invertir para principiantes México | fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -815,12 +819,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AsesorÃ­a Financiera para Mujeres en MÃ©xico | Eunik</t>
+          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://regcheq.com.mx/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -830,24 +834,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en MÃ©xico a travÃ©s de asesorÃ­a especializada en inversiones, enfocÃ¡ndonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/regcheqmx/</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/regcheqmexico/</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>contactomx@regcheq.com</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -858,12 +870,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -873,28 +885,28 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>tu@email.com</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | fintech inversión Argentina principiantes</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -905,12 +917,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://regcheq.com.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -920,32 +932,28 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/regcheqmx/</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/regcheqmexico/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>contactomx@regcheq.com</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -956,43 +964,43 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Principales noticias de Colombia y el mundo | La FM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.lafm.com.co/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Entérate de las noticias de Colombia y el mundo al instante. Información de última hora, verificada, análisis y opinión. Mantente bien informado cada día.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lafmoficial/</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>contacto@lakpa.lat</t>
-        </is>
-      </c>
+          <t>https://co.linkedin.com/company/rcnradio</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -1003,43 +1011,39 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>hello@capitellefinance.com</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -1050,47 +1054,43 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Forbes Argentina</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.forbesargentina.com/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Forbes Argentina | La marca número 1 de negocios del mundo en Argentina.</t>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/forbesargentina/</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://ar.linkedin.com/company/forbes-argentina</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>swiper@7.0.5, vanilla-lazyload@12.4.0</t>
+          <t>info@bolsa24.com</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1152,86 +1152,86 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
-        </is>
-      </c>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>18d2f96d279149989b95faf0a4b41882@sentry-next.wixpress.com, 2062d0a4929b45348643784b5cb39c36@sentry.wixpress.com, 5d1795a2db124a268f1e1bd88f503500@sentry.wixpress.com</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+          <t>Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1242,51 +1242,55 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Mercadopeso🥇Compara préstamos y tarjetas de crédito</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://www.mercadopeso.mx/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1296,319 +1300,839 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Mercadopeso México es una empresa de comparación de préstamos y tarjetas de crédito ✅ Mercadopeso es confiable para las mejores opciones y ofertas financieras 🤑</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>info@mercadopeso.mx</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NameResolu</t>
-        </is>
-      </c>
+          <t>app para invertir para principiantes México</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Latinas Invest â Money, Investing and Ownership for Latina Women</t>
+          <t>Inversión Familiar — Educación financiera para familias</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.latinasinvest.com/</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://inversionfamiliar.es/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Investing education by and for Latinas: why the wealth gap exists, how to start investing with what you have, the women to learn from, and how Latinasâ¦</t>
+          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>info@inversionfamiliar.es</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>https://finan.mx/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx, ejemplo@correo.com, nombre@ejemplo.com</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mujeres inversionistas | UBS México</t>
+          <t>Flink – Venture Capital</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.ubs.com/</t>
+          <t>https://flink.co/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>inversion, mujeres, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión. Estamos aquí para guiar tu empresa hacia el éxito con nuestra experiencia y dedicación.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flink-co/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>info@flink.co</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
-        </is>
-      </c>
+          <t>Flink app inversión</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>InversiÃ³n MÃ¡s Rentable | Trading AlgorÃ­tmico e IA Financiera | InversiÃ³n MÃ¡s Rentable</t>
+          <t>Inversiones Chidas | Inversiones y Educación Financiera</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>https://inversioneschidas.com/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Expertos en trading algorÃ­tmico, inteligencia artificial para inversiones y consultorÃ­a financiera. Maximiza tus rendimientos con tecnologÃ­a de punta.</t>
+          <t>Aprende como invertir con guías paso a paso y material 100% gratis para formarte en temas de inversiones y educación financiera en México.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com, wght@400..800</t>
-        </is>
-      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>GBM+ inversión | GBM+ inversión</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Home - GBM</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://about.appgbm.com/</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>https://www.mujeresinvirtiendo.com/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/gbmplus_/</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/gbm-mx</t>
-        </is>
-      </c>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NameResolu</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>53</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DineroenImagen</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.dineroenimagen.com/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>slick-carousel@1.8.1</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>fintech inversión mujeres Latinoamérica</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>53</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>53</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Diario de Trading con IA para Traders | Awake Trader | Awake Trader</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.awaketrader.com/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Diario de trading con IA que audita tus emociones y mejora tu disciplina. Mentor IA, backtesting y sistema de consistencia. Garantía de reembolso de 14 días.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://instagram.com/awaketrader.app</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>hola@awaketrader.com, legal@awaketrader.com, privacidad@awaketrader.com</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>53</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://fintual.mx/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Fintual | Fintual</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>53</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Microwd Inversiones - genera impacto social</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/microwd_inv/</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>info@microwd.es, name@email.es, wght@300..700</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Microwd | Microwd</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>53</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Microwd 2026 Company Profile: Valuation, Funding &amp; Investors ...MICROWD - Products, Competitors, Financials, Employees ...Microwd - Facebook</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://pitchbook.com/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, principiantes, digital</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Operator of a fintech platform intended to facilitate investment in microcredit projects for women entrepreneurs. The company connects investors with borrowers and lists loan projects across sectors such as agriculture, retail, and services, enabling women to receive financing for their businesses. Want detailed data on 11M+ companies? Jul 27, 2023 · MICROWD is a fintech company that focuses on impact investing within the financial services sector. The company provides a platform for investors to fund microloans to women entrepreneurs in Latin America. Jun 12, 2026 · Nuevo sistema MICROWD Estrenamos plataforma: más clara, más segura y con nuevo diseño. Invertir ahora es más sencillo y tu experiencia mejora desde el primer clic. 👉 Importante: para entrar por primera vez solo tendrás que recuperar tu contraseña.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Microwd</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://pitchbook.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>47</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ADDEM CAPITAL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.addemcapital.mx/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, mujeres, latam</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Su producto Pilou Kids permite a las familias abrir cuentas de inversión para menores de edad, con los padres como cotitulares. Cuando el niño o la niña cumple 18 años, la cuenta pasa a su nombre, fomentando desde la infancia una conversación abierta y sana sobre el manejo del dinero.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/addem_capital/</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/addem-capital/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>usuario@dominio.com</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>47</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | fintech inversión Argentina principiantes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>41</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com, wght@400..800</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>41</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>http://caraneco.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>502 Server Error: Bad Gateway for url: http://caraneco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>41</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>GBM+ inversión</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>41</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Home - GBM</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://about.appgbm.com/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, digital</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gbmplus_/</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gbm-mx</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K26"/>
+  <autoFilter ref="A1:K38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-17
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,46 +500,54 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PRO Network</t>
+          <t>Mujeres y Dinero | educación financiera</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.pronetwork.mx/</t>
+          <t>https://www.mujeres-y-dinero.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujeresydinerouy/</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/mujeresydinero/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>contanos@mujeresydinero.uy</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -589,7 +597,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -600,17 +608,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -618,74 +626,78 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>educación financiera para mujeres invertir startup | Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/visionarias.business/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/visionarias</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -696,12 +708,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>PRO Network</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://www.pronetwork.mx/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -714,28 +726,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>contacto@asesoresinversion.com</t>
-        </is>
-      </c>
+          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero | fintech mexicana para invertir desde poco dinero | app de ahorro e inversión México jóvenes</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -746,17 +754,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -769,23 +777,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fintual/</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>luisdrive57@gmail.com</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -796,66 +800,58 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Morado Inclusive Fintech 2024 Nuestra Misión Impulsamos negocios, transformamos futuros En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>fintech mexicana para invertir desde poco dinero | app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -868,40 +864,44 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.finamex.com.mx/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -914,24 +914,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -942,12 +946,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -960,28 +964,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -992,163 +992,171 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Microwd - Nicaragua</t>
+          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://microwdnicaragua.com/</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>https://regcheq.com.mx/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>mujeres, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Financiamos los negocios de las mujeres más extraordinarias de Nicaragua</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/regcheqmx/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/regcheqmexico/</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>oficina1.nica@microwd.es, oficina2.nica@microwd.es</t>
+          <t>contactomx@regcheq.com</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Microwd</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>servicioal.cliente@puntored.co</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>info@bolsa24.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Escuela profesional de traders - NovatosTrading Club</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://www.novatostradingclub.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1156,224 +1164,216 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+          <t>Escuela Profesional de Traders con más de 11 años de experiencia formando traders ganadores. Aprende a ganar dinero en Bolsa.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/novatos.trading.club/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="b">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Capitelle Finance</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>hello@capitellefinance.com</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Flink – Venture Capital</t>
+          <t>Microwd - Nicaragua</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://flink.co/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://microwdnicaragua.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="b">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
+          <t>mujeres, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión.</t>
+          <t>Financiamos los negocios de las mujeres más extraordinarias de Nicaragua</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/flink-co/</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>info@flink.co</t>
+          <t>oficina1.nica@microwd.es, oficina2.nica@microwd.es</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Flink app inversión</t>
+          <t>Microwd</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NameResolu</t>
-        </is>
-      </c>
+          <t>fintech inversión Argentina principiantes | fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
-        </is>
-      </c>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Mujer Emprende</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://www.mujeremprendeglobal.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1386,96 +1386,116 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+          <t>Escuela de Negocios para Mujeres</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujeremprendeglobal</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mujer-emprende/</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E22" t="b">
         <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1483,321 +1503,313 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>info@bolsa24.com</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://fmaartini.cl/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>Franco Martini</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://kuspit.com/</t>
+          <t>https://www.inversionmasrentable.com/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, principiantes, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>fintech inversión Argentina principiantes | GBM+ inversión | GBM+ inversión</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Microwd Inversiones - genera impacto social</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.microwd.es/</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>https://fundacionana.org/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
       <c r="E27" t="b">
         <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Microwd | Microwd</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ADDEM CAPITAL</t>
+          <t>Educación Financiera e Inversión Inteligente para Crecer -</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.addemcapital.mx/</t>
+          <t>https://hazcrecereldinero.com/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>En México, más de 10 millones de mujeres han vivido violencia económica, pero menos del 13% la reconoce», afirma Patricia Florencia, cofundadora de Pilou.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/addem_capital/</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/addem-capital/</t>
-        </is>
-      </c>
+          <t>Aprende a invertir, ahorrar y generar ingresos pasivos con guías claras y estrategias reales. Tu libertad financiera empieza aquí, sin rodeos.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
         <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1805,23 +1817,23 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ahorro Rinde -</t>
+          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://ahorrorinde.com.mx/</t>
+          <t>https://www.bbva.mx/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1834,12 +1846,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1847,23 +1859,23 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>startup mexicana inversión patrimonial personas | startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
+          <t>Finanzas Transparentes | Finsus</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://akibaa.com/</t>
+          <t>https://finsus.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1876,66 +1888,62 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+          <t>SOFIPO líder en México, especializada en ahorro e inversión con rendimientos competitivos y total seguridad. Abre tu cuenta en minutos y haz crecer tu dinero de forma simple, confiable y sin complicaciones.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/finsusapp</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+          <t>info@finsus.mx</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cómo invertir en Perú siendo principiante: desde S/100</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, principiantes, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 · El mercado de inversión en Perú se ha democratizado con plataformas digitales que permiten invertir desde S/100. Esta guía muestra el camino desde el depósito a plazo hasta los fondos indexados globales.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1943,45 +1951,41 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>403 Client Error: Forbidden for url: https://cashcontrolly.com/</t>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NameResolu</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Guías de Viaje</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://guiasdeviaje.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="b">
         <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1989,13 +1993,680 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>53</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Información sobre negocios financieros en México</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://negociosfinancieros.com.mx/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>53</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://apartadomex.com.mx/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>53</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://godinmx.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E36" t="b">
+        <v>1</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>app de ahorro e inversión México jóvenes</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>53</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.finfit.mx/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>53</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://kuspit.com/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Kuspit | Kuspit</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>53</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Microwd Inversiones - genera impacto social</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="b">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/microwd_inv/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>info@microwd.es</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Microwd | Microwd</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>47</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, mujeres, digital</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>47</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>47</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://marketb2b.mx/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>47</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>47</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Tappoyo, la fintech peruana que transforma la vida de las mujeres</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://frecuenciamoney.com/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>0</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, latam, digital</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Sep 23, 2024 · A través de implementaciones tecnológicas, Tappoyo realiza análisis alternativos del perfil crediticio de las usuarias Más del 70% de las mujeres que reciben estos créditos son madres solteras, y 3 de cada 10 han iniciado un nuevo emprendimiento tras recibir financiamiento Se convirtió en la primera fintech en Latinoamérica en desembolsar préstamos grupales a mujeres en zonas rurales ...</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Tappoyo Perú</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>47</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Microwd 2026 Company Profile: Valuation, Funding &amp; Investors ...Microwd Inversiones - LinkedInMicrowd - México</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://pitchbook.com/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, latam, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Information on valuation, funding, cap tables, investors, and executives for Microwd. Use the PitchBook Platform to explore the full profile. Microwd Inversiones | 2,868 followers on LinkedIn. |M. The fintech for the unbanked. | Microwd is a fintech that connects women entrepreneurs in Latin America who want a microloan with investors ... Microwd es una organización que ofrece microcréditos individuales a partir de 3,000 MXN a mujeres que quieren iniciar o mejorar su negocio en México. Conoce su historia, equipo, impacto y preguntas frecuentes.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Microwd</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://pitchbook.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>47</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Microwd - México</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://microwd.mx/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, asesoria, latam</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Microwd en México</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Microwd</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>41</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cómo invertir en Perú siendo principiante: desde S/100</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://cashcontrolly.com/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>0</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, latam, digital</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Feb 20, 2026 · El mercado de inversión en Perú se ha democratizado con plataformas digitales que permiten invertir desde S/100. Esta guía muestra el camino desde el depósito a plazo hasta los fondos indexados globales.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://cashcontrolly.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>41</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L33"/>
+  <autoFilter ref="A1:L48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-18
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,54 +500,46 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mujeres y Dinero | educación financiera</t>
+          <t>Tandazo — Autofinanciamiento $50k a $220k MXN sin intereses ni buró</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.mujeres-y-dinero.com/</t>
+          <t>https://tandazo.com.mx/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/mujeresydinerouy/</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujeresydinero/</t>
-        </is>
-      </c>
+          <t>Mensualidad fija $2,500 MXN. Sin historial crediticio, sin aval. Comprueba solo capacidad de pago. 100% digital.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>contanos@mujeresydinero.uy</t>
+          <t>contratos@tandazo.com.mx, privacidad@tandazo.com.mx</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -597,7 +589,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -608,17 +600,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -626,28 +618,28 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup | Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -658,12 +650,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -681,69 +673,73 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
+          <t>https://www.instagram.com/fundssociety/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
+          <t>https://www.linkedin.com/company/funds-society/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PRO Network</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.pronetwork.mx/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -754,21 +750,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -777,19 +773,23 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -800,21 +800,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -823,19 +823,19 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+          <t>luisdrive57@gmail.com</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero | app de ahorro e inversión México jóvenes</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -846,12 +846,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -869,39 +869,35 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.finamex.com.mx/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -914,28 +910,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -946,12 +938,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -964,24 +956,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>hola@eunik.mx</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para principiantes Perú | fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -992,12 +984,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://regcheq.com.mx/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1015,22 +1007,18 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/regcheqmx/</t>
-        </is>
-      </c>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/regcheqmexico/</t>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>contactomx@regcheq.com</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1046,12 +1034,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1064,28 +1052,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>contacto@lakpa.lat</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1096,21 +1084,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1119,44 +1107,44 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>info@bolsa24.com</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Escuela profesional de traders - NovatosTrading Club</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.novatostradingclub.com/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1164,179 +1152,203 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Escuela Profesional de Traders con más de 11 años de experiencia formando traders ganadores. Aprende a ganar dinero en Bolsa.</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/novatos.trading.club/</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://capitellefinance.com/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>https://www.yotepresto.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/yotepresto-com</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>hello@capitellefinance.com</t>
+          <t>info@yotepresto.com</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Microwd - Nicaragua</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://microwdnicaragua.com/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>https://www.tappoyo.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
       <c r="E17" t="b">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>mujeres, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Financiamos los negocios de las mujeres más extraordinarias de Nicaragua</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>oficina1.nica@microwd.es, oficina2.nica@microwd.es</t>
-        </is>
-      </c>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Microwd</t>
+          <t>Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+          <t>https://www.instagram.com/finan.mx/</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes | fintech mexicana para invertir desde poco dinero</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.teiainvest.co/</t>
+          <t>https://fmaartini.cl/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1344,12 +1356,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1357,23 +1369,23 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mujer Emprende</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.mujeremprendeglobal.com/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1386,98 +1398,82 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Escuela de Negocios para Mujeres</t>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujeremprendeglobal</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujer-emprende/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1490,12 +1486,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1503,28 +1499,32 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Latinas Invest — Money, Investing and Ownership for Latina Women</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://www.latinasinvest.com/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1532,326 +1532,306 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
+          <t>Investing education by and for Latinas: why the wealth gap exists, how to start investing with what you have, the women to learn from, and how Latinas…</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>info@bolsa24.com</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>Información sobre negocios financieros en México</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
+          <t>https://negociosfinancieros.com.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes | GBM+ inversión | GBM+ inversión</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://godinmx.com/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Educación Financiera e Inversión Inteligente para Crecer -</t>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://hazcrecereldinero.com/</t>
+          <t>https://losbancos.mx/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Aprende a invertir, ahorrar y generar ingresos pasivos con guías claras y estrategias reales. Tu libertad financiera empieza aquí, sin rodeos.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Fondos de Inversión en Monterrey | Planes Planifica Futuro</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
+          <t>https://www.planificafuturo.com/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>Fondos y planes de inversión en Monterrey Nuevo León. Asesor especialista con 12 años de experiencia atención personalizada para asegurar tu futuro financiero con la experiencia de Planifica Futuro.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/planificafuturo/</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.bbva.mx/</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="b">
         <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1859,23 +1839,27 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas | startup mexicana inversión patrimonial personas</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Finanzas Transparentes | Finsus</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://finsus.mx/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1888,62 +1872,50 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>SOFIPO líder en México, especializada en ahorro e inversión con rendimientos competitivos y total seguridad. Abre tu cuenta en minutos y haz crecer tu dinero de forma simple, confiable y sin complicaciones.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finsusapp</t>
-        </is>
-      </c>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>info@finsus.mx</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Guadalajara fintech inversión ahorro</t>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Home - Conade IP</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://conadeip.mx/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="b">
         <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Posts Populares: Recientes:</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1951,41 +1923,41 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NameResolu</t>
-        </is>
-      </c>
+          <t>asesor de inversión independiente registrado CNBV</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Ahorro Rinde -</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>https://ahorrorinde.com.mx/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E33" t="b">
         <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1993,129 +1965,129 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>contacto@apartadomex.com.mx</t>
+          <t>contacto@inversionmasrentable.com</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Cómo invertir en Perú siendo principiante: desde S/100</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://cashcontrolly.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+          <t>Feb 20, 2026 · El mercado de inversión en Perú se ha democratizado con plataformas digitales que permiten invertir desde S/100. Esta guía muestra el camino desde el depósito a plazo hasta los fondos indexados globales.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2123,69 +2095,69 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
+          <t>plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://cashcontrolly.com/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>10 startups latinoamericanas que apuestan por la equidad género</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.caf.com/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Mujeres WOW: Plataforma de fondos colaborativos para financiar negocios liderados por mujeres. Mujeres WOW nació bajo el compromiso de brindar soluciones financieras para las pequeñas empresas lideradas por mujeres.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.caf.com', port=443): Max retries exceeded with url: / (Caused by SSLError(SSLCertVerificat</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Guías de Viaje</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://kuspit.com/</t>
+          <t>https://guiasdeviaje.mx/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2198,12 +2170,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, principiantes, asesoria, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -2211,462 +2183,13 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>53</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Microwd Inversiones - genera impacto social</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://www.microwd.es/</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="b">
-        <v>0</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Microwd | Microwd</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>47</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, mujeres, digital</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>47</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>https://mifinguia.com/</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E41" t="b">
-        <v>1</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>47</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>https://marketb2b.mx/</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E42" t="b">
-        <v>1</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>47</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Puntored</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>https://puntored.mx/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E43" t="b">
-        <v>1</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>47</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Tappoyo, la fintech peruana que transforma la vida de las mujeres</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://frecuenciamoney.com/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
-      <c r="E44" t="b">
-        <v>0</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, latam, digital</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Sep 23, 2024 · A través de implementaciones tecnológicas, Tappoyo realiza análisis alternativos del perfil crediticio de las usuarias Más del 70% de las mujeres que reciben estos créditos son madres solteras, y 3 de cada 10 han iniciado un nuevo emprendimiento tras recibir financiamiento Se convirtió en la primera fintech en Latinoamérica en desembolsar préstamos grupales a mujeres en zonas rurales ...</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Tappoyo Perú</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>47</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Microwd 2026 Company Profile: Valuation, Funding &amp; Investors ...Microwd Inversiones - LinkedInMicrowd - México</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://pitchbook.com/</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E45" t="b">
-        <v>1</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, latam, digital</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Information on valuation, funding, cap tables, investors, and executives for Microwd. Use the PitchBook Platform to explore the full profile. Microwd Inversiones | 2,868 followers on LinkedIn. |M. The fintech for the unbanked. | Microwd is a fintech that connects women entrepreneurs in Latin America who want a microloan with investors ... Microwd es una organización que ofrece microcréditos individuales a partir de 3,000 MXN a mujeres que quieren iniciar o mejorar su negocio en México. Conoce su historia, equipo, impacto y preguntas frecuentes.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Microwd</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://pitchbook.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>47</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Microwd - México</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://microwd.mx/</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E46" t="b">
-        <v>1</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>mujeres, educacion, asesoria, latam</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Microwd en México</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Microwd</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>41</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Cómo invertir en Perú siendo principiante: desde S/100</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://cashcontrolly.com/</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
-      <c r="E47" t="b">
-        <v>0</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>inversion, principiantes, latam, digital</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Feb 20, 2026 · El mercado de inversión en Perú se ha democratizado con plataformas digitales que permiten invertir desde S/100. Esta guía muestra el camino desde el depósito a plazo hasta los fondos indexados globales.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para principiantes Perú</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://cashcontrolly.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>GBMfondos</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L48"/>
+  <autoFilter ref="A1:L38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-19
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -504,163 +504,163 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tandazo — Autofinanciamiento $50k a $220k MXN sin intereses ni buró</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://tandazo.com.mx/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mensualidad fija $2,500 MXN. Sin historial crediticio, sin aval. Comprueba solo capacidad de pago. 100% digital.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>contratos@tandazo.com.mx, privacidad@tandazo.com.mx</t>
-        </is>
-      </c>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://finantres.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/finantres/</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>contacto@finantres.com</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>contacto@asesoresinversion.com</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -668,49 +668,49 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundssociety/</t>
+          <t>https://www.instagram.com/fintual/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
+          <t>https://www.linkedin.com/company/fintual/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E6" t="b">
@@ -718,44 +718,48 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>Morado Inclusive Fintech 2024 Nuestra Misión Impulsamos negocios, transformamos futuros En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/moradocolombia/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>contacto@morado.app</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -768,90 +772,94 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>hola@eunik.mx</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero | fintech mexicana para invertir desde poco dinero</t>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Mujeres en Finanzas</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://www.mujeresenfinanzas.mx/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>Tan solo en México, la participación igualitaria podría representar un crecimiento de hasta 70% del PIB nacional, de acuerdo a la Asociación de Mujeres Jefas de Empresas (AMMJE). Si las mujeres participaran de forma igualitaria a nivel global, esto podría agregar al PIB entre 13% y 31% para 2025.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujeresenfinanzas/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mujeres-en-finanzas-m%C3%A9xico</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>info@mujeresenfinanzas.mx</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -864,24 +872,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México | plataforma para invertir en CETES y ETFs México</t>
+          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -892,12 +900,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -910,24 +918,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -938,12 +950,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Inicio - ASEM - Asociación de Emprendedores de México</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://asem.mx/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -956,90 +968,102 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Haciendo de México el mejor lugar para emprender y hacer negocios</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+          <t>https://www.instagram.com/asem_socios</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/asem-mx</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>info@asem.mx</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para principiantes Perú | fintech inversión Argentina principiantes</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+          <t>https://www.linkedin.com/company/puntored/</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://becasbenitojuarezmx.com/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1052,78 +1076,74 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETFs, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://inv.mx/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>https://www.instagram.com/invierteenseguros/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invseguros</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>info@bolsa24.com</t>
+          <t>contacto@inv.mx</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1134,17 +1154,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1152,132 +1172,112 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
+          <t>https://www.instagram.com/tappoyofintech/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
+          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.yotepresto.com/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://mente-mujer.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
+          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/yotepresto-com</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>info@yotepresto.com</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://www.bbva.mx/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
+          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú</t>
+          <t>app de ahorro e inversión México jóvenes | startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1288,46 +1288,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="b">
         <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>atencion.al.cliente@finan.mx</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1338,17 +1326,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Flink – Venture Capital</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://flink.co/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1356,36 +1344,44 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flink-co/</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>info@flink.co</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>Flink app inversión</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1398,58 +1394,54 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.kuspit.com/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="b">
         <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1457,7 +1449,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -1468,45 +1460,49 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finxard/</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1514,38 +1510,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Latinas Invest — Money, Investing and Ownership for Latina Women</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.latinasinvest.com/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Investing education by and for Latinas: why the wealth gap exists, how to start investing with what you have, the women to learn from, and how Latinas…</t>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -1556,26 +1556,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Información sobre negocios financieros en México</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>https://negociosfinancieros.com.mx/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E24" t="b">
         <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1583,7 +1587,7 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -1594,12 +1598,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://godinmx.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1612,24 +1616,20 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1640,12 +1640,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1658,20 +1658,24 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1682,12 +1686,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://fintual.mx/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1700,20 +1704,28 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -1724,17 +1736,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://losbancos.mx/</t>
+          <t>https://www.inversionmasrentable.com/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E28" t="b">
@@ -1747,35 +1759,35 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
-        </is>
-      </c>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Fondos de Inversión en Monterrey | Planes Planifica Futuro</t>
+          <t>Emprende Pro Mujer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.planificafuturo.com/</t>
+          <t>https://emprendepromujer.org/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1784,24 +1796,20 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Fondos y planes de inversión en Monterrey Nuevo León. Asesor especialista con 12 años de experiencia atención personalizada para asegurar tu futuro financiero con la experiencia de Planifica Futuro.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/planificafuturo/</t>
-        </is>
-      </c>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
@@ -1812,26 +1820,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E30" t="b">
         <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1839,14 +1851,10 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1854,12 +1862,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Chatterize - Get the best financial products on the market</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://chatterize.com/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1872,12 +1880,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+          <t>Get the best financial products on the market</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1885,7 +1893,7 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
@@ -1896,26 +1904,30 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Home - Conade IP</t>
+          <t>Ahorro Rinde -</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://conadeip.mx/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>https://ahorrorinde.com.mx/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E32" t="b">
         <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Posts Populares: Recientes:</t>
+          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1923,7 +1935,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
@@ -1934,12 +1946,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ahorro Rinde -</t>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://ahorrorinde.com.mx/</t>
+          <t>https://marketb2b.mx/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1952,12 +1964,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1965,53 +1977,62 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Puntored</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://puntored.mx/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
@@ -2022,41 +2043,45 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>Mujeres inversionistas | UBS México</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>https://www.ubs.com/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria</t>
+          <t>inversion, mujeres, latam</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2064,17 +2089,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cómo invertir en Perú siendo principiante: desde S/100</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
+          <t>http://caraneco.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E36" t="b">
@@ -2082,12 +2107,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, principiantes, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 · El mercado de inversión en Perú se ha democratizado con plataformas digitales que permiten invertir desde S/100. Esta guía muestra el camino desde el depósito a plazo hasta los fondos indexados globales.</t>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2095,12 +2120,12 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>403 Client Error: Forbidden for url: https://cashcontrolly.com/</t>
+          <t>502 Server Error: Bad Gateway for url: http://caraneco.com/</t>
         </is>
       </c>
     </row>
@@ -2110,41 +2135,49 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10 startups latinoamericanas que apuestan por la equidad género</t>
+          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.caf.com/</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>https://activeleasing.mx/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, mujeres, digital</t>
+          <t>inversion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Mujeres WOW: Plataforma de fondos colaborativos para financiar negocios liderados por mujeres. Mujeres WOW nació bajo el compromiso de brindar soluciones financieras para las pequeñas empresas lideradas por mujeres.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/activeleasing/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.caf.com', port=443): Max retries exceeded with url: / (Caused by SSLError(SSLCertVerificat</t>
-        </is>
-      </c>
+          <t>inversión como prestación para empleados México fintech</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2188,8 +2221,192 @@
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>41</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://ecosistemastartup.com/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>hola@ecosistemastartup.com</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>startup mexicana inversión patrimonial personas</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>41</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>41</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Home - GBM</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://about.appgbm.com/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, digital</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gbmplus_/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gbm-mx</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Home | QED Investors</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.qedinvestors.com/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>At Morado we are building a next generation B2B marketplace for the beauty and wellness industry, the everything store for beauty shops. We provide access to thousands of products at great prices, and offer an end-to-end solution, from access to credit and equipment rentals, to last mile logistics. In Latam, women account for 84% of the beauty industry workforce and our mission is to enable ...</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/qed-investors/</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Morado fintech Colombia</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
+  <autoFilter ref="A1:L42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-20
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Mujeres y Dinero | educación financiera</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://www.mujeres-y-dinero.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,145 +522,153 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/mujeresydinerouy/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/mujeresydinero/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>contanos@mujeresydinero.uy</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundssociety/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | app de ahorro e inversión México jóvenes</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://finantres.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/finantres/</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>contacto@finantres.com</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -668,28 +676,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -700,21 +708,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>PRO Network</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://www.pronetwork.mx/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -723,43 +731,35 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Morado Inclusive Fintech 2024 Nuestra Misión Impulsamos negocios, transformamos futuros En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
+          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>contacto@morado.app</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -772,40 +772,40 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mujeres en Finanzas</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.mujeresenfinanzas.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -818,128 +818,128 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, empresas_b2b, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Tan solo en México, la participación igualitaria podría representar un crecimiento de hasta 70% del PIB nacional, de acuerdo a la Asociación de Mujeres Jefas de Empresas (AMMJE). Si las mujeres participaran de forma igualitaria a nivel global, esto podría agregar al PIB entre 13% y 31% para 2025.</t>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujeresenfinanzas/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujeres-en-finanzas-m%C3%A9xico</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>info@mujeresenfinanzas.mx</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>luisdrive57@gmail.com</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/moradocolombia/</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>contacto@morado.app</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -950,12 +950,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Inicio - ASEM - Asociación de Emprendedores de México</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://asem.mx/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -968,53 +968,45 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Haciendo de México el mejor lugar para emprender y hacer negocios</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asem_socios</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/asem-mx</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>info@asem.mx</t>
+          <t>hola@eunik.mx</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>BioBioChile - La Red de Prensa Más Grande de Chile</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.biobiochile.cl/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1022,29 +1014,25 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>La Red de Prensa Más Grande de Chile</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
+          <t>https://www.instagram.com/biobiochile/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/biobiochile/</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>fintech inversión mujeres Latinoamérica</t>
@@ -1054,16 +1042,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1076,36 +1064,40 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
+          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://inv.mx/</t>
+          <t>https://regcheq.com.mx/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1118,140 +1110,148 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
+          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/invierteenseguros/</t>
+          <t>https://www.instagram.com/regcheqmx/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/invseguros</t>
+          <t>https://www.linkedin.com/company/regcheqmexico/</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>contacto@inv.mx</t>
+          <t>contactomx@regcheq.com</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>contacto@lakpa.lat</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://mente-mujer.com/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>https://www.el-fondo.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
       <c r="E16" t="b">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
-        </is>
-      </c>
+          <t>plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
+          <t>Trámites en México explicados paso a paso | Conade IP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.bbva.mx/</t>
+          <t>https://conadeip.mx/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1264,12 +1264,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+          <t>Requisitos, costos 2026 y pasos de pasaporte, RFC, CURP, IMSS, actas y licencias. Guía independiente con checklist de documentos y enlace a la fuente oficial.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1277,61 +1277,77 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes | startup mexicana inversión patrimonial personas</t>
+          <t>asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>https://puntored.co/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Flink – Venture Capital</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://flink.co/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1344,44 +1360,36 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión.</t>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/flink-co/</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>info@flink.co</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Flink app inversión</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://www.yotepresto.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1394,54 +1402,62 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/yotepresto-com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>info@yotepresto.com</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>app de ahorro e inversión México jóvenes</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E21" t="b">
         <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1449,359 +1465,359 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
+          <t>FinTech in Mexico — Inteligencia FinTech México</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://finxard.com/</t>
+          <t>https://www.fintechinmexico.com/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finxard/</t>
-        </is>
-      </c>
+          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>contacto@finxard.com, johndoe@gmail.com</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>contacto@apartadomex.com.mx</t>
+          <t>info@bolsa24.com</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
+          <t>https://www.inversionmasrentable.com/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>contacto@finfit.mx</t>
+          <t>contacto@inversionmasrentable.com</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>fintech inversión Argentina principiantes | GBM+ inversión</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="b">
         <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer</t>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>https://marketb2b.mx/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1809,41 +1825,41 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>7 Mejores - Comparativas para elegir con acierto</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://7mejores.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, mujeres, asesoria, empresas_b2b, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+          <t>Encuentra comparativas y recomendaciones de los mejores productos y servicios. Toma decisiones informadas con nuestras guías actualizadas.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1851,23 +1867,23 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chatterize - Get the best financial products on the market</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://chatterize.com/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1880,36 +1896,40 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Get the best financial products on the market</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ahorro Rinde -</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://ahorrorinde.com.mx/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1922,12 +1942,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1935,41 +1955,41 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://marketb2b.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="b">
         <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1977,78 +1997,65 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Puntored</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://puntored.mx/</t>
+          <t>https://cashcontrolly.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mujeres inversionistas | UBS México</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.ubs.com/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2061,58 +2068,58 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, mujeres, latam</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
-        </is>
-      </c>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+          <t>Información sobre negocios financieros en México</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>http://caraneco.com/</t>
+          <t>https://negociosfinancieros.com.mx/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2120,27 +2127,23 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>502 Server Error: Bad Gateway for url: http://caraneco.com/</t>
-        </is>
-      </c>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://activeleasing.mx/</t>
+          <t>https://godinmx.com/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2153,44 +2156,36 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/activeleasing/</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
-        </is>
-      </c>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>inversión como prestación para empleados México fintech</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Guías de Viaje</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://guiasdeviaje.mx/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2203,41 +2198,45 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://ecosistemastartup.com/</t>
+          <t>https://losbancos.mx/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E39" t="b">
@@ -2245,62 +2244,58 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>hola@ecosistemastartup.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>GBMfondos</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>https://kuspit.com/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+          <t>inversion, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Información sobre fondos de inversión GBM</t>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2308,105 +2303,542 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Home - GBM</t>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca ...</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://about.appgbm.com/</t>
+          <t>https://heraldodemexico.com.mx/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, digital</t>
+          <t>inversion, ahorro, mujeres, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/gbmplus_/</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/gbm-mx</t>
-        </is>
-      </c>
+          <t>Apr 17, 2023 · Andrea de la Garza y Patricia Florencia son las creadoras de Pilou, la primera plataforma de ahorro e inversión creada por mujeres, pensada para mujeres</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Home | QED Investors</t>
+          <t>EMPRENDE PRO MUJER</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://www.qedinvestors.com/</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>At Morado we are building a next generation B2B marketplace for the beauty and wellness industry, the everything store for beauty shops. We provide access to thousands of products at great prices, and offer an end-to-end solution, from access to credit and equipment rentals, to last mile logistics. In Latam, women account for 84% of the beauty industry workforce and our mission is to enable ...</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/qed-investors/</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia</t>
+          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>47</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>47</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Finec México</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://finec.com.mx/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>FINEC Asset Management, S.A. de C.V., Asesor en Inversiones Independiente registrado ante la CNBV. Asesoría patrimonial independiente con visión de largo plazo en México.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>jmateos@finec.com.mx</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>asesor de inversión independiente registrado CNBV</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>47</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ahorro Rinde -</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://ahorrorinde.com.mx/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>47</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Tappoyo, la fintech peruana que transforma la vida de las mujeres</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://frecuenciamoney.com/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>0</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, latam, digital</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Sep 23, 2024 · A través de implementaciones tecnológicas, Tappoyo realiza análisis alternativos del perfil crediticio de las usuarias Más del 70% de las mujeres que reciben estos créditos son madres solteras, y 3 de cada 10 han iniciado un nuevo emprendimiento tras recibir financiamiento Se convirtió en la primera fintech en Latinoamérica en desembolsar préstamos grupales a mujeres en zonas rurales ...</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Tappoyo Perú</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>41</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://activeleasing.mx/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inversion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/activeleasing/</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>inversión como prestación para empleados México fintech</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://finaipedia.com/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, latam, digital</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://bitso.com/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>41</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Guías de Viaje</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://guiasdeviaje.mx/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>41</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L42"/>
+  <autoFilter ref="A1:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-21
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -608,17 +608,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://finantres.com/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -626,78 +626,78 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/finantres/</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera para mujeres invertir startup | Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>contacto@asesoresinversion.com</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>plataforma de inversión para mujeres México | asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -708,42 +708,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PRO Network</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.pronetwork.mx/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>luisdrive57@gmail.com</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -754,58 +754,66 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/moradocolombia/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+          <t>contacto@morado.app</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>DeDinero</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://www.dedinero.com.mx/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -818,128 +826,120 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
+          <t>Noticias de dinero de última hora de México y el mundo.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>daniel.fitta@elgrafico.mx, francisco.perez@clabsa.com.mx, itzelnavarrete@correocpn.com.mx</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>luisdrive57@gmail.com</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión para mujeres México | app para invertir para principiantes México | fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -950,63 +950,63 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Inversiones24: Tu Portal de Confianza para Invertir desde Latinoamérica</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://www.inversiones24.com/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+          <t>Descubre en Inversiones24 las mejores plataformas de inversión, brokers regulados, cursos y guías para aprender a invertir en bolsa, acciones, ETF y criptomonedas.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>info@colonna-global-media.com</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BioBioChile - La Red de Prensa Más Grande de Chile</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.biobiochile.cl/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1014,25 +1014,29 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>La Red de Prensa Más Grande de Chile</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/biobiochile/</t>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/biobiochile/</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>fintech inversión mujeres Latinoamérica</t>
@@ -1042,171 +1046,163 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Principales noticias de Colombia y el mundo | La FM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.lafm.com.co/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Entérate de las noticias de Colombia y el mundo al instante. Información de última hora, verificada, análisis y opinión. Mantente bien informado cada día.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>https://www.instagram.com/lafmoficial/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://co.linkedin.com/company/rcnradio</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | fintech inversión Argentina principiantes</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PLD México 2026: Software y Cumplimiento Antilavado | Regcheq</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://regcheq.com.mx/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>PLD en México: la plataforma líder para Entidades Financieras y Actividades Vulnerables. Cumple LFPIORPI y DCG con KYC, monitoreo y reportes automatizados a la UIF y el SAT.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/regcheqmx/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/regcheqmexico/</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>contactomx@regcheq.com</t>
-        </is>
-      </c>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>contacto@lakpa.lat</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1214,145 +1210,137 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+          <t>https://www.linkedin.com/company/colcapital</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Trámites en México explicados paso a paso | Conade IP</t>
+          <t>Inversión Familiar — Educación financiera para familias</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://conadeip.mx/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://inversionfamiliar.es/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Requisitos, costos 2026 y pasos de pasaporte, RFC, CURP, IMSS, actas y licencias. Guía independiente con checklist de documentos y enlace a la fuente oficial.</t>
+          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>info@inversionfamiliar.es</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>servicioal.cliente@puntored.co</t>
+          <t>atencion.al.cliente@finan.mx</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.teiainvest.co/</t>
+          <t>https://fmaartini.cl/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1360,12 +1348,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1373,115 +1361,111 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
+          <t>EconomiaeInversion.com - Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.yotepresto.com/</t>
+          <t>https://economiaeinversion.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
+          <t>Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/yotepresto-com</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>info@yotepresto.com</t>
-        </is>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FinTech in Mexico — Inteligencia FinTech México</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.fintechinmexico.com/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1494,12 +1478,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1507,123 +1491,111 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Asesoría financiera para mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, asesoria, latam</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones para mujeres. Nuestro enfoque moderno y minimalista busca empoderar a las mujeres en su camino hacia la independencia financiera.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>info@bolsa24.com</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Kuspit</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='eunik.mx', port=443): Max retries exceeded with url: / (Caused by NewConnectionError("HTTPSCon</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1636,132 +1608,136 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finxard/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>contacto@inversionmasrentable.com</t>
+          <t>contacto@apartadomex.com.mx</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes | GBM+ inversión</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
+          <t>https://heraldodemexico.com.mx/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1770,12 +1746,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, ahorro, mujeres, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
+          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -1783,41 +1759,41 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+          <t>Emprende Pro Mujer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://marketb2b.mx/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1825,41 +1801,41 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>7 Mejores - Comparativas para elegir con acierto</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://7mejores.com/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, mujeres, asesoria, empresas_b2b, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Encuentra comparativas y recomendaciones de los mejores productos y servicios. Toma decisiones informadas con nuestras guías actualizadas.</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1867,23 +1843,23 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Puntored</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
+          <t>https://puntored.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1896,100 +1872,109 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, educacion, asesoria</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas | fintech inversión Argentina principiantes | GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>http://caraneco.com/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1997,65 +1982,77 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>HTTPConnectionPool(host='caraneco.com', port=80): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
+          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
+          <t>https://activeleasing.mx/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/activeleasing/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>inversión como prestación para empleados México fintech</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://bitso.com/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2068,21 +2065,25 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>fintech mexicana para invertir desde poco dinero</t>
@@ -2092,16 +2093,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://finaipedia.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2114,12 +2115,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2134,16 +2135,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2156,689 +2157,68 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>Monterrey fintech inversión personas | Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>GBMfondos</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="b">
         <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Información sobre fondos de inversión GBM</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
     </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>53</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://losbancos.mx/</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E39" t="b">
-        <v>1</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Monterrey fintech inversión personas</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>53</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://kuspit.com/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E40" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>inversion, principiantes, asesoria, latam, digital</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Kuspit | Kuspit</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>47</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca ...</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="b">
-        <v>1</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, mujeres, digital</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Apr 17, 2023 · Andrea de la Garza y Patricia Florencia son las creadoras de Pilou, la primera plataforma de ahorro e inversión creada por mujeres, pensada para mujeres</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>47</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>EMPRENDE PRO MUJER</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="b">
-        <v>0</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, educacion</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>47</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>https://mifinguia.com/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E43" t="b">
-        <v>1</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>47</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Finec México</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://finec.com.mx/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E44" t="b">
-        <v>1</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, asesoria, regulada, latam</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>FINEC Asset Management, S.A. de C.V., Asesor en Inversiones Independiente registrado ante la CNBV. Asesoría patrimonial independiente con visión de largo plazo en México.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>jmateos@finec.com.mx</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>47</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Ahorro Rinde -</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://ahorrorinde.com.mx/</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E45" t="b">
-        <v>1</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>47</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Puntored</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://puntored.mx/</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E46" t="b">
-        <v>1</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>47</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Tappoyo, la fintech peruana que transforma la vida de las mujeres</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://frecuenciamoney.com/</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
-      <c r="E47" t="b">
-        <v>0</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, latam, digital</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Sep 23, 2024 · A través de implementaciones tecnológicas, Tappoyo realiza análisis alternativos del perfil crediticio de las usuarias Más del 70% de las mujeres que reciben estos créditos son madres solteras, y 3 de cada 10 han iniciado un nuevo emprendimiento tras recibir financiamiento Se convirtió en la primera fintech en Latinoamérica en desembolsar préstamos grupales a mujeres en zonas rurales ...</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Tappoyo Perú</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://activeleasing.mx/</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E48" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>inversion, asesoria, latam, digital</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/activeleasing/</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>inversión como prestación para empleados México fintech</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>41</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>https://finaipedia.com/</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E49" t="b">
-        <v>1</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>inversion, principiantes, latam, digital</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>41</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>https://bitso.com/</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E50" t="b">
-        <v>1</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>41</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Guías de Viaje</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://guiasdeviaje.mx/</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E51" t="b">
-        <v>1</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>41</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>GBMfondos</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="b">
-        <v>1</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L52"/>
+  <autoFilter ref="A1:L38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-22
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mujeres y Dinero | educación financiera</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.mujeres-y-dinero.com/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,53 +522,49 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujeresydinerouy/</t>
+          <t>https://www.instagram.com/fundssociety/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujeresydinero/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>contanos@mujeresydinero.uy</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -576,28 +572,28 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundssociety/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -608,17 +604,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -626,28 +622,28 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup | Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -658,12 +654,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -681,23 +677,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -708,21 +700,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -731,19 +723,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -754,17 +750,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -772,78 +768,74 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>luisdrive57@gmail.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DeDinero</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.dedinero.com.mx/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Noticias de dinero de última hora de México y el mundo.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>daniel.fitta@elgrafico.mx, francisco.perez@clabsa.com.mx, itzelnavarrete@correocpn.com.mx</t>
-        </is>
-      </c>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintual/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -854,12 +846,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -872,24 +864,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | app para invertir para principiantes México | fintech inversión Argentina principiantes</t>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -900,12 +892,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -918,28 +910,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>contacto@lakpa.lat</t>
-        </is>
-      </c>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>plataforma de inversión para mujeres México | app para invertir para principiantes México | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -950,63 +938,67 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Inversiones24: Tu Portal de Confianza para Invertir desde Latinoamérica</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.inversiones24.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Descubre en Inversiones24 las mejores plataformas de inversión, brokers regulados, cursos y guías para aprender a invertir en bolsa, acciones, ETF y criptomonedas.</t>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>info@colonna-global-media.com</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1014,103 +1006,95 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Principales noticias de Colombia y el mundo | La FM</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.lafm.com.co/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="b">
         <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Entérate de las noticias de Colombia y el mundo al instante. Información de última hora, verificada, análisis y opinión. Mantente bien informado cada día.</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/lafmoficial/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://co.linkedin.com/company/rcnradio</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>hello@capitellefinance.com</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.teiainvest.co/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1118,20 +1102,28 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>info@bolsa24.com</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1142,17 +1134,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1160,44 +1152,48 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1210,82 +1206,86 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Inversión Familiar — Educación financiera para familias</t>
+          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://inversionfamiliar.es/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>https://www.yotepresto.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
+          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/yotepresto-com</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>info@inversionfamiliar.es</t>
+          <t>info@yotepresto.com</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://becasbenitojuarezmx.com/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1298,91 +1298,87 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>atencion.al.cliente@finan.mx</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://misfinanzasdigitales.com/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EconomiaeInversion.com - Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://economiaeinversion.com/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1390,20 +1386,28 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1414,104 +1418,100 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
+          <t>https://mente-mujer.com/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="b">
         <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
+          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>fintech inversión mujeres Latinoamérica</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Asesoría financiera para mujeres en México | Eunik</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1524,54 +1524,62 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, mujeres, asesoria, latam</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones para mujeres. Nuestro enfoque moderno y minimalista busca empoderar a las mujeres en su camino hacia la independencia financiera.</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='eunik.mx', port=443): Max retries exceeded with url: / (Caused by NewConnectionError("HTTPSCon</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>https://fmaartini.cl/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1579,28 +1587,28 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://finxard.com/</t>
+          <t>https://www.inversionmasrentable.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -1608,216 +1616,220 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finxard/</t>
-        </is>
-      </c>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>contacto@finxard.com, johndoe@gmail.com</t>
+          <t>contacto@inversionmasrentable.com</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>fintech inversión Argentina principiantes | GBM+ inversión</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="b">
         <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>https://www.posta.com.mx/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E28" t="b">
         <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
+          <t>Monterrey fintech inversión personas</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer</t>
+          <t>Flink – Venture Capital</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>https://flink.co/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E29" t="b">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión. Estamos aquí para guiar tu empresa hacia el éxito con nuestra experiencia y dedicación.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flink-co/</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>info@flink.co</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
+          <t>Flink app inversión</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1830,12 +1842,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1843,23 +1855,23 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Puntored</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://puntored.mx/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1872,109 +1884,100 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>https://www.dineroenimagen.com/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | fintech inversión Argentina principiantes | GBM+ inversión</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>http://caraneco.com/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -1982,77 +1985,73 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>HTTPConnectionPool(host='caraneco.com', port=80): Read timed out. (read timeout=15)</t>
-        </is>
-      </c>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Active Leasing :: Take it easy. Take it Leasing.</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://activeleasing.mx/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Aug 28, 2026 · Las inversiones a través de plataformas fintech pueden generar intereses sujetos a obligaciones fiscales. Conoce qué impuestos pueden aplicar, cómo funcionan las retenciones y qué aspectos deben considerar las personas físicas en México durante 2026.</t>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/activeleasing/</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/active-leasing-s-a-de-c-v</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+          <t>https://www.instagram.com/finxard/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>inversión como prestación para empleados México fintech</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://bitso.com/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2065,25 +2064,21 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>fintech mexicana para invertir desde poco dinero</t>
@@ -2093,16 +2088,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://finaipedia.com/</t>
+          <t>https://godinmx.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2115,12 +2110,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, principiantes, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2128,23 +2123,23 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2157,68 +2152,859 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas | Monterrey fintech inversión personas</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GBMfondos</t>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>https://losbancos.mx/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E38" t="b">
         <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
+          <t>Monterrey fintech inversión personas</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>53</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://fintual.mx/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Fintual | Fintual</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>53</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Microwd Inversiones - genera impacto social</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/microwd_inv/</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>info@microwd.es</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Microwd | Microwd</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>47</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, mujeres, digital</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>47</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>47</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Simulador de Credito Hipotecario Mexico 2026 — CotizadorHipotecario.mx</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://cotizadorhipotecario.mx/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Simulador de credito hipotecario gratuito para Mexico. Calcula tu mensualidad, CAT, tabla de amortizacion, gastos notariales. Compara bancos: BBVA, Banorte, Santander. Mas de 100 calculadoras financieras.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>inversión como prestación para empleados México fintech</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>47</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Ahorro Rinde -</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://ahorrorinde.com.mx/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>47</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://marketb2b.mx/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>47</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://akibaa.com/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>41</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Mujeres inversionistas | UBS México</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.ubs.com/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, latam</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>http://caraneco.com/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E49" t="b">
+        <v>0</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Investment Management &amp; Financial Services | BlackRock</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.blackrock.com/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>0</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/blackrock</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>41</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CashControlly · End the month with money, not red numbers</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://cashcontrolly.com/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>0</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>41</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://finaipedia.com/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, latam, digital</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>41</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://bitso.com/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>41</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Cronista Usa - El Cronista</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.cronista.com/</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E54" t="b">
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>El Cronista es uno de los Diarios Económicos de Argentina más valoraEs la fuente más confiable de información sobre Economía, Finanzas y Negocios.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cronistacom</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/cronistacom/</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>atencionalcliente@cronista.com, atroiano@cronista.com, bpersico@cronista.com</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Guadalajara fintech inversión ahorro</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>41</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
           <t>GBM+ inversión</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
+  <autoFilter ref="A1:L55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-23
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Mujeres y Dinero | educación financiera</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://www.mujeres-y-dinero.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,28 +522,32 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundssociety/</t>
+          <t>https://www.instagram.com/mujeresydinerouy/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/mujeresydinero/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>contanos@mujeresydinero.uy</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -593,7 +597,7 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup | Mujer Financiera Argentina</t>
+          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -650,46 +654,50 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundssociety/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras | Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -700,21 +708,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -723,23 +731,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>luisdrive57@gmail.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -750,17 +754,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -768,74 +772,82 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/moradocolombia/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>contacto@morado.app</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>contacto@asesoresinversion.com</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -846,42 +858,46 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>hola@eunik.mx</t>
-        </is>
-      </c>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -892,113 +908,117 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>hello@capitellefinance.com</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | app para invertir para principiantes México | plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+          <t>https://www.linkedin.com/company/puntored/</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1006,328 +1026,316 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para principiantes Perú | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>MEMIVI – Mejorando mi vida</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://capitellefinance.com/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>https://memivi.mx/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>Descubre cómo comenzar a invertir en México con poco dinero, utilizando herramientas accesibles, estrategias prácticas y pasos claros que te permitan hacer crecer tu capital sin asumir riesgos innecesarios desde el inicio.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>hello@capitellefinance.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/memivi.oficial/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://br.linkedin.com/company/jbf-digital-marketing</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://www.yotepresto.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/yotepresto-com</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>info@bolsa24.com</t>
+          <t>info@yotepresto.com</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://mente-mujer.com/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="b">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
+          <t>Inversión Familiar — Educación financiera para familias</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.teiainvest.co/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://inversionfamiliar.es/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="b">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
+          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>info@inversionfamiliar.es</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
+          <t>Burcamp</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.yotepresto.com/</t>
+          <t>https://burcamp.co/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/yotepresto-com</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>info@yotepresto.com</t>
-        </is>
-      </c>
+          <t>Burcamp</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/burcamp/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://misfinanzasdigitales.com/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1340,233 +1348,225 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
-        </is>
-      </c>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, asesoria, latam</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://eunik.mx/</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://mente-mujer.com/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>https://www.dineroenimagen.com/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
-        </is>
-      </c>
+          <t>fintech inversión mujeres Latinoamérica</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>InversionPasiva ▷▷ Invertir bien nunca fue tan fácil</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://inversionpasiva.es/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="b">
         <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+          <t>Todo sobre el ahorro, la inversión pasiva en fondos indexados y el camino a seguir para alcanzar la independencia financiera.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/finan.mx/</t>
+          <t>https://www.instagram.com/finxard/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>atencion.al.cliente@finan.mx</t>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Invierte en acciones, fondos, ETFs y renta fija en Colombia - trii</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://trii.co/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1574,41 +1574,49 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+          <t>trii es la plataforma para invertir en Bolsa de Valores, fondos, ETFs y renta fija en Colombia. Comisión más baja, sin papeleo y todo desde tu celular. Segura y fácil.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/somostrii/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/somostrii/mycompany/</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
+          <t>https://cashcontrolly.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -1616,86 +1624,82 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes | GBM+ inversión</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
+          <t>https://softcredito.com.mx/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1704,12 +1708,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1717,23 +1721,23 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1746,108 +1750,104 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Flink – Venture Capital</t>
+          <t>Microwd Inversiones - genera impacto social</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://flink.co/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
+          <t>inversion, mujeres, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión. Estamos aquí para guiar tu empresa hacia el éxito con nuestra experiencia y dedicación.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/microwd_inv/</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/flink-co/</t>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>info@flink.co</t>
+          <t>info@microwd.es</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Flink app inversión</t>
+          <t>Microwd | Microwd</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Emprende Pro Mujer</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.kuspit.com/</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1855,23 +1855,23 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1884,12 +1884,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1897,27 +1897,23 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Puntored</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://puntored.mx/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1930,83 +1926,108 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>https://akibaa.com/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E33" t="b">
         <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
+          <t>Cronista Usa - El Cronista</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://finxard.com/</t>
+          <t>https://www.cronista.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Estados Unidos</t>
         </is>
       </c>
       <c r="E34" t="b">
@@ -2014,44 +2035,48 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+          <t>El Cronista es uno de los Diarios Económicos de Argentina más valoraEs la fuente más confiable de información sobre Economía, Finanzas y Negocios.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/finxard/</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>https://www.instagram.com/cronistacom</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/cronistacom/</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>contacto@finxard.com, johndoe@gmail.com</t>
+          <t>atencionalcliente@cronista.com, atroiano@cronista.com, bpersico@cronista.com</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Mujeres inversionistas | UBS México</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://www.ubs.com/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2064,128 +2089,128 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, latam</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>contacto@finfit.mx</t>
+          <t>contacto@inversionmasrentable.com</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://losbancos.mx/</t>
+          <t>http://caraneco.com/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2194,44 +2219,44 @@
         </is>
       </c>
       <c r="E38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
-        </is>
-      </c>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://bitso.com/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2244,767 +2269,176 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintualmx/</t>
+          <t>https://instagram.com/bitso</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
+          <t>https://www.linkedin.com/company/bitso</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Microwd Inversiones - genera impacto social</t>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.microwd.es/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>https://marketb2b.mx/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
+          <t>educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Microwd | Microwd</t>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca dar a las ...</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>https://www.posta.com.mx/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E41" t="b">
         <v>1</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Con 27 años en el sector financiero, Patricia y Andrea decidieron llevar sus conocimientos a más personas, "manejamos portafolios de inversión para clientes que tienen arriba de un millón de dólares y trabajando en esta institución nos dimos cuenta de varias cosas, la principal que sigue siendo un sector extremadamente liderado por hombres y que además son muy pocas las mujeres que ...</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
+          <t>Monterrey fintech inversión personas</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://ecosistemastartup.com/</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>hola@ecosistemastartup.com</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+          <t>Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>47</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Simulador de Credito Hipotecario Mexico 2026 — CotizadorHipotecario.mx</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>https://cotizadorhipotecario.mx/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E43" t="b">
-        <v>1</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, asesoria, latam, digital</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Simulador de credito hipotecario gratuito para Mexico. Calcula tu mensualidad, CAT, tabla de amortizacion, gastos notariales. Compara bancos: BBVA, Banorte, Santander. Mas de 100 calculadoras financieras.</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>inversión como prestación para empleados México fintech</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>47</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Ahorro Rinde -</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://ahorrorinde.com.mx/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E44" t="b">
-        <v>1</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>47</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://marketb2b.mx/</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E45" t="b">
-        <v>1</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>47</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://akibaa.com/</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E46" t="b">
-        <v>1</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>47</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Puntored</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://puntored.mx/</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E47" t="b">
-        <v>1</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>41</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Mujeres inversionistas | UBS México</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://www.ubs.com/</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E48" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, latam</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>41</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>http://caraneco.com/</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E49" t="b">
-        <v>0</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>41</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Investment Management &amp; Financial Services | BlackRock</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>https://www.blackrock.com/</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E50" t="b">
-        <v>0</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/blackrock</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>41</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://cashcontrolly.com/</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="E51" t="b">
-        <v>0</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>41</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>FinAIpedia - Compara Préstamos Rápidos en México | Tu Mejor Opción Financiera</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>https://finaipedia.com/</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E52" t="b">
-        <v>1</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>inversion, principiantes, latam, digital</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Compara los mejores préstamos rápidos en línea en México. Encuentra tasas bajas, aprobación rápida y dinero en minutos. ¡Solicita tu préstamo hoy con FinAIpedia!</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>41</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>https://bitso.com/</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E53" t="b">
-        <v>1</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>41</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Cronista Usa - El Cronista</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>https://www.cronista.com/</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="E54" t="b">
-        <v>0</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>El Cronista es uno de los Diarios Económicos de Argentina más valoraEs la fuente más confiable de información sobre Economía, Finanzas y Negocios.</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/cronistacom</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/cronistacom/</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>atencionalcliente@cronista.com, atroiano@cronista.com, bpersico@cronista.com</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Guadalajara fintech inversión ahorro</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>41</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>GBMfondos</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="b">
-        <v>1</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L55"/>
+  <autoFilter ref="A1:L42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-24
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mujeres y Dinero | educación financiera</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.mujeres-y-dinero.com/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,32 +522,28 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujeresydinerouy/</t>
+          <t>https://www.instagram.com/fundssociety/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujeresydinero/</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>contanos@mujeresydinero.uy</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -558,17 +554,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -576,28 +572,28 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -608,17 +604,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -626,78 +622,74 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>PRO Network</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://www.pronetwork.mx/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundssociety/</t>
-        </is>
-      </c>
+          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
+          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras | Monterrey fintech inversión personas</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -708,21 +700,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -731,19 +723,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -754,17 +750,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E7" t="b">
@@ -772,82 +768,74 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>luisdrive57@gmail.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>contacto@asesoresinversion.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fintual/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -858,46 +846,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>app para invertir para principiantes México | fintech inversión Argentina principiantes | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -908,63 +892,67 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://capitellefinance.com/</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>https://lakpa.mx/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>hello@capitellefinance.com</t>
+          <t>contacto@lakpa.lat</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -972,53 +960,49 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>servicioal.cliente@puntored.co</t>
+          <t>info@bolsa24.com</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Inversiones24: Tu Portal de Confianza para Invertir desde Latinoamérica</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.inversiones24.com/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E12" t="b">
@@ -1026,74 +1010,66 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
+          <t>Descubre en Inversiones24 las mejores plataformas de inversión, brokers regulados, cursos y guías para aprender a invertir en bolsa, acciones, ETF y criptomonedas.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>info@colonna-global-media.com</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú | fintech mexicana para invertir desde poco dinero</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MEMIVI – Mejorando mi vida</t>
+          <t>Microwd - Nicaragua</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://memivi.mx/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://microwdnicaragua.com/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
+          <t>mujeres, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Descubre cómo comenzar a invertir en México con poco dinero, utilizando herramientas accesibles, estrategias prácticas y pasos claros que te permitan hacer crecer tu capital sin asumir riesgos innecesarios desde el inicio.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/memivi.oficial/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://br.linkedin.com/company/jbf-digital-marketing</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+          <t>Financiamos los negocios de las mujeres más extraordinarias de Nicaragua</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>oficina1.nica@microwd.es, oficina2.nica@microwd.es</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>Microwd</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1104,151 +1080,163 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.yotepresto.com/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/yotepresto-com</t>
+          <t>https://www.linkedin.com/company/puntored/</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>info@yotepresto.com</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
+          <t>Revista Emprendedores | Portada</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://mente-mujer.com/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>https://emprendedores.es/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
       <c r="E15" t="b">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+          <t>Portada de la Revista Emprendedores.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
-        </is>
-      </c>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Inversión Familiar — Educación financiera para familias</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://inversionfamiliar.es/</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>info@inversionfamiliar.es</t>
-        </is>
-      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Burcamp</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://burcamp.co/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -1256,24 +1244,28 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Burcamp</t>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/burcamp/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1284,17 +1276,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -1307,35 +1299,35 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1348,58 +1340,62 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>EconomiaeInversion.com - Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://economiaeinversion.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, asesoria, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+          <t>Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1407,27 +1403,23 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://eunik.mx/</t>
-        </is>
-      </c>
+          <t>fintech inversión Argentina principiantes</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://www.bbva.mx/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1440,54 +1432,50 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
-        </is>
-      </c>
+          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>InversionPasiva ▷▷ Invertir bien nunca fue tan fácil</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://inversionpasiva.es/</t>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Todo sobre el ahorro, la inversión pasiva en fondos indexados y el camino a seguir para alcanzar la independencia financiera.</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1495,141 +1483,129 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://finxard.com/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/finxard/</t>
+          <t>https://www.instagram.com/postamx/</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>contacto@finxard.com, johndoe@gmail.com</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Invierte en acciones, fondos, ETFs y renta fija en Colombia - trii</t>
+          <t>FinTech in Mexico — Inteligencia FinTech México</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://trii.co/</t>
+          <t>https://www.fintechinmexico.com/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>trii es la plataforma para invertir en Bolsa de Valores, fondos, ETFs y renta fija en Colombia. Comisión más baja, sin papeleo y todo desde tu celular. Segura y fácil.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/somostrii/</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/somostrii/mycompany/</t>
-        </is>
-      </c>
+          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1637,7 +1613,7 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1648,12 +1624,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1666,27 +1642,27 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>contacto@apartadomex.com.mx</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1694,26 +1670,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Asesoría financiera para mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>https://eunik.mx/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E27" t="b">
         <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, mujeres, asesoria, latam</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones para mujeres. Nuestro enfoque moderno y minimalista busca empoderar a las mujeres en su camino hacia la independencia financiera.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1721,10 +1701,14 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='eunik.mx', port=443): Max retries exceeded with url: / (Caused by NewConnectionError("HTTPSCon</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1732,12 +1716,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
+          <t>https://www.dineroenimagen.com/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1750,24 +1734,24 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -1778,142 +1762,146 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Microwd Inversiones - genera impacto social</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.microwd.es/</t>
+          <t>https://softcredito.com.mx/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Microwd | Microwd</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer</t>
+          <t>InvestSmart México — Asesoría de inversiones independiente</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>https://isasesoria.mx/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
       <c r="E30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>inversion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+          <t>Impulsamos personas para que vivan sus mejores oportunidades. Asesoría de inversiones independiente en México, con la fuerza de un grupo de más de 100 oficinas.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>contacto@investsmart.com.mx</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | educación financiera para mujeres invertir startup</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Invierte en acciones, fondos, ETFs y renta fija en Colombia - trii</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://trii.co/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+          <t>trii es la plataforma para invertir en Bolsa de Valores, fondos, ETFs y renta fija en Colombia. Comisión más baja, sin papeleo y todo desde tu celular. Segura y fácil.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/somostrii/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/somostrii/mycompany/</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Puntored</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://puntored.mx/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1926,429 +1914,429 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>53</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://godinmx.com/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>app de ahorro e inversión México jóvenes</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>53</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PAN CDMX</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.pancdmx.org.mx/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, educacion, latam</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Sitio Oficial del PAN CDMX. Partido Acción Nacional en la Ciudad de México.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pan_cdmx/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>estudios.pancmx@gmail.com</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>educación financiera e inversión para mujeres CDMX</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>53</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.finfit.mx/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>53</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://ecosistemastartup.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="E36" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>hola@ecosistemastartup.com</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Guadalajara fintech inversión ahorro | Guadalajara fintech inversión ahorro</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>53</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://fintual.mx/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Fintual | Fintual</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>53</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Microwd Inversiones - genera impacto social</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/microwd_inv/</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>info@microwd.es</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Microwd | Microwd</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>47</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>47</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>inversion, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Somos la red transaccional  que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>https://www.instagram.com/puntoredmx/</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>contacto@gestopago.com, contacto@puntored.mx</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>47</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>https://akibaa.com/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E33" t="b">
-        <v>1</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>47</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Cronista Usa - El Cronista</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://www.cronista.com/</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Estados Unidos</t>
-        </is>
-      </c>
-      <c r="E34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, asesoria, latam, digital</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>El Cronista es uno de los Diarios Económicos de Argentina más valoraEs la fuente más confiable de información sobre Economía, Finanzas y Negocios.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/cronistacom</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/cronistacom/</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>atencionalcliente@cronista.com, atroiano@cronista.com, bpersico@cronista.com</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Guadalajara fintech inversión ahorro</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>41</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Mujeres inversionistas | UBS México</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>https://www.ubs.com/</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E35" t="b">
-        <v>1</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, latam</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>41</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>https://colcapital.org/</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E36" t="b">
-        <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>41</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="b">
-        <v>0</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>inversion, educacion, asesoria</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>roboadvisor México carteras diversificadas</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>41</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>http://caraneco.com/</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E38" t="b">
-        <v>0</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>41</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>https://bitso.com/</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E39" t="b">
-        <v>1</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>41</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>https://marketb2b.mx/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E40" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>educacion, asesoria, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
+          <t>https://akibaa.com/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2361,24 +2349,32 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
@@ -2389,17 +2385,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://ecosistemastartup.com/</t>
+          <t>http://caraneco.com/</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E42" t="b">
@@ -2412,33 +2408,193 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>hola@ecosistemastartup.com</t>
-        </is>
-      </c>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Guadalajara fintech inversión ahorro</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Investment Management &amp; Financial Services | BlackRock</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.blackrock.com/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/blackrock</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CashControlly · End the month with money, not red numbers</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://cashcontrolly.com/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>0</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="b">
+        <v>0</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L42"/>
+  <autoFilter ref="A1:L46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-25
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,16 +500,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -522,28 +522,28 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundssociety/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -554,17 +554,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -572,78 +572,74 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -654,12 +650,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PRO Network</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.pronetwork.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -672,24 +668,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Impulsamos la prosperidad empresarial con tecnología, reconocimiento y bienestar organizacional</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/3836753/admin/dashboard/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>contacto@asesoresinversion.com</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -700,142 +700,142 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>https://www.instagram.com/moradocolombia/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>contacto@asesoresinversion.com</t>
+          <t>contacto@morado.app</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>hola@eunik.mx</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -846,12 +846,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -864,24 +864,28 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>contacto@lakpa.lat</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech inversión Argentina principiantes | fintech mexicana para invertir desde poco dinero</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -892,67 +896,67 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>info@bolsa24.com</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E11" t="b">
@@ -960,44 +964,48 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>info@bolsa24.com</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inversiones24: Tu Portal de Confianza para Invertir desde Latinoamérica</t>
+          <t>Revista Emprendedores | Portada</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.inversiones24.com/</t>
+          <t>https://emprendedores.es/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1010,66 +1018,70 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Descubre en Inversiones24 las mejores plataformas de inversión, brokers regulados, cursos y guías para aprender a invertir en bolsa, acciones, ETF y criptomonedas.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>info@colonna-global-media.com</t>
-        </is>
-      </c>
+          <t>Portada de la Revista Emprendedores.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Microwd - Nicaragua</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://microwdnicaragua.com/</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>mujeres, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Financiamos los negocios de las mujeres más extraordinarias de Nicaragua</t>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>oficina1.nica@microwd.es, oficina2.nica@microwd.es</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Microwd</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1080,116 +1092,100 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://misfinanzasdigitales.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Revista Emprendedores | Portada</t>
+          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://emprendedores.es/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
+          <t>https://mente-mujer.com/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="b">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Portada de la Revista Emprendedores.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
-        </is>
-      </c>
+          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Mercadopeso🥇Compara préstamos y tarjetas de crédito</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://www.mercadopeso.mx/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1202,70 +1198,74 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
+          <t>Mercadopeso México es una empresa de comparación de préstamos y tarjetas de crédito ✅ Mercadopeso es confiable para las mejores opciones y ofertas financieras 🤑</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>info@mercadopeso.mx</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>app para invertir para principiantes México</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -1276,42 +1276,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1322,12 +1314,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://marketb2b.mx/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1340,28 +1332,20 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>atencion.al.cliente@finan.mx</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -1372,17 +1356,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EconomiaeInversion.com - Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
+          <t>Flink – Venture Capital</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://economiaeinversion.com/</t>
+          <t>https://flink.co/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1390,20 +1374,28 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Noticias y actualidad en Economía, Inversión, Finanzas y Mercado Inmobiliario</t>
+          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión. Estamos aquí para guiar tu empresa hacia el éxito con nuestra experiencia y dedicación.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flink-co/</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>info@flink.co</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>Flink app inversión</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1414,12 +1406,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.bbva.mx/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1432,12 +1424,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1445,37 +1437,41 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>https://www.mujeresinvirtiendo.com/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E22" t="b">
         <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1483,74 +1479,70 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="b">
         <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FinTech in Mexico — Inteligencia FinTech México</t>
+          <t>InvestSmart México — Asesoría de inversiones independiente</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.fintechinmexico.com/</t>
+          <t>https://isasesoria.mx/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1558,36 +1550,40 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+          <t>Impulsamos personas para que vivan sus mejores oportunidades. Asesoría de inversiones independiente en México, con la fuerza de un grupo de más de 100 oficinas.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>contacto@investsmart.com.mx</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Guadalajara fintech inversión ahorro</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Información sobre negocios financieros en México</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.kuspit.com/</t>
+          <t>https://negociosfinancieros.com.mx/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1600,12 +1596,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1613,7 +1609,7 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1624,12 +1620,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://apartadomex.com.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1642,27 +1638,27 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1670,12 +1666,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Asesoría financiera para mujeres en México | Eunik</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1688,27 +1684,27 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, mujeres, asesoria, latam</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones para mujeres. Nuestro enfoque moderno y minimalista busca empoderar a las mujeres en su camino hacia la independencia financiera.</t>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='eunik.mx', port=443): Max retries exceeded with url: / (Caused by NewConnectionError("HTTPSCon</t>
-        </is>
-      </c>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1716,12 +1712,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Plataforma de Beneficios Para Empleados | minu</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://www.minu.mx/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1734,54 +1730,58 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+          <t>Fideliza y atrae al mejor talento en tu empresa con los beneficios para empleados más valorados. Minu la mejor forma de compensar a tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/minuservicios/posts/?feedView=all</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sergio.godinez@minu.mx</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Emprende Pro Mujer</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
+          <t>https://emprendepromujer.org/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1789,28 +1789,28 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>InvestSmart México — Asesoría de inversiones independiente</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://isasesoria.mx/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E30" t="b">
@@ -1818,90 +1818,78 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Impulsamos personas para que vivan sus mejores oportunidades. Asesoría de inversiones independiente en México, con la fuerza de un grupo de más de 100 oficinas.</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>contacto@investsmart.com.mx</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Invierte en acciones, fondos, ETFs y renta fija en Colombia - trii</t>
+          <t>Ahorro Rinde -</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://trii.co/</t>
+          <t>https://ahorrorinde.com.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>trii es la plataforma para invertir en Bolsa de Valores, fondos, ETFs y renta fija en Colombia. Comisión más baja, sin papeleo y todo desde tu celular. Segura y fácil.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/somostrii/</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/somostrii/mycompany/</t>
-        </is>
-      </c>
+          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://akibaa.com/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1914,40 +1902,48 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>contacto@apartadomex.com.mx</t>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Puntored</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://puntored.mx/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1960,36 +1956,49 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PAN CDMX</t>
+          <t>Mujeres inversionistas | UBS México</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.pancdmx.org.mx/</t>
+          <t>https://www.ubs.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2002,95 +2011,91 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, mujeres, latam</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Sitio Oficial del PAN CDMX. Partido Acción Nacional en la Ciudad de México.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/pan_cdmx/</t>
-        </is>
-      </c>
+          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>estudios.pancmx@gmail.com</t>
-        </is>
-      </c>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
+          <t>http://manesseco.com/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia . Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://ecosistemastartup.com/</t>
+          <t>http://www.caraneco.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E36" t="b">
@@ -2098,166 +2103,150 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>hola@ecosistemastartup.com</t>
-        </is>
-      </c>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia . Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Guadalajara fintech inversión ahorro | Guadalajara fintech inversión ahorro</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://www.caraneco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://trocaco.com/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia . Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Microwd Inversiones - genera impacto social</t>
+          <t>Sanineco | Educación Financiera en Colombia</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.microwd.es/</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>http://sanineco.com/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E38" t="b">
         <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
+          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia . Plataforma líder en análisis de mercados e información económica colombiana.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Microwd | Microwd</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Bureaco | Educación Financiera en Colombia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>http://bureaco.com/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2265,119 +2254,106 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Puntored</t>
+          <t>Ramenesco - Educación Financiera en Colombia</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://puntored.mx/</t>
+          <t>http://www.ramenesco.com/</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
+          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia . Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras .</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://www.ramenesco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
+          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://akibaa.com/</t>
+          <t>http://larednco.com/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
-        </is>
-      </c>
+          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia . Descubre estrategias de inversión y mejora tu futuro financiero.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2385,21 +2361,21 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>http://caraneco.com/</t>
+          <t>https://bitso.com/</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2408,22 +2384,26 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
-        </is>
-      </c>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2431,170 +2411,40 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Investment Management &amp; Financial Services | BlackRock</t>
+          <t>GBMfondos</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.blackrock.com/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
+          <t>Información sobre fondos de inversión GBM</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/blackrock</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L43" t="inlineStr"/>
     </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>41</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://cashcontrolly.com/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="E44" t="b">
-        <v>0</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para principiantes Chile</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>41</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>GBMfondos</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="b">
-        <v>1</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="b">
-        <v>0</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>inversion, educacion, asesoria</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>contacto@inversionmasrentable.com</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L46"/>
+  <autoFilter ref="A1:L43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-26
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Perfil | Ultimas noticias de Argentina y el mundo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.perfil.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,28 +522,24 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
+          <t>Periodismo Puro: breaking news, análisis y los mejores columnistas cubriendo los temas más importantes de la Argentina y el mundo</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/perfilcom/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -554,17 +550,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://finantres.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -572,124 +568,128 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
-        </is>
-      </c>
+          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/finantres/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>contacto@finantres.com</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/visionarias.business/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/visionarias</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>contacto@asesoresinversion.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
+          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -700,158 +700,146 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>En Morado, creemos en el poder de las oportunidades. Nuestra misión es brindar acceso a soluciones financieras ágiles y flexibles que impulsen el crecimiento de emprendedores y negocios en Colombia y Latinoamérica.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://comparabancaperu.com/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>luisdrive57@gmail.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Bolsa de Chile | IPSA en Tiempo Real | Portal #1 de Inversiones</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.bolsadechile.cl/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
+          <t>Cotizaciones IPSA, dólar, UF y fondos mutuos en tiempo real. Educación financiera, calculadoras y comunidad de inversores chilenos. Tu portal financiero de referencia.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://www.finamex.com.mx/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -864,49 +852,49 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>contacto@lakpa.lat</t>
-        </is>
-      </c>
+          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -914,44 +902,44 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>info@bolsa24.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fintual/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -964,98 +952,94 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
+          <t>https://www.instagram.com/moradocolombia/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>servicioal.cliente@puntored.co</t>
+          <t>contacto@morado.app</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Revista Emprendedores | Portada</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://emprendedores.es/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Portada de la Revista Emprendedores.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1068,36 +1052,40 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://misfinanzasdigitales.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1110,308 +1098,344 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>contacto@lakpa.lat</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://mente-mujer.com/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>https://asesoresinversion.com/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>contacto@asesoresinversion.com</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas | plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mercadopeso🥇Compara préstamos y tarjetas de crédito</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.mercadopeso.mx/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mercadopeso México es una empresa de comparación de préstamos y tarjetas de crédito ✅ Mercadopeso es confiable para las mejores opciones y ofertas financieras 🤑</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>info@mercadopeso.mx</t>
-        </is>
-      </c>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>atencion.al.cliente@finan.mx</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>Inicio - BlockIT Lab</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
+          <t>https://blockitlab.com/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>El laboratorio donde suceden tus ideas</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/blockitlab/</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>proyectos@blockitlab.com</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+          <t>Revista Emprendedores | Portada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://marketb2b.mx/</t>
+          <t>https://emprendedores.es/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+          <t>Portada de la Revista Emprendedores.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Flink – Venture Capital</t>
+          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://flink.co/</t>
+          <t>https://www.yotepresto.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión. Estamos aquí para guiar tu empresa hacia el éxito con nuestra experiencia y dedicación.</t>
+          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/flink-co/</t>
+          <t>https://www.linkedin.com/company/yotepresto-com</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>info@flink.co</t>
+          <t>info@yotepresto.com</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Flink app inversión</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.kuspit.com/</t>
+          <t>https://inv.mx/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1424,125 +1448,149 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/invierteenseguros/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invseguros</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>contacto@inv.mx</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>Startups Argentina — Directorio y trabajos en el ecosistema startup</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://www.startupsargentina.com/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
+          <t>Explorá startups de Argentina, LATAM y Estados Unidos que contratan talento desde Argentina.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>karen@yafu.app, people@tapi.la</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>Mujer Financiera Argentina</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>https://www.tappoyo.com/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
       <c r="E23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>InvestSmart México — Asesoría de inversiones independiente</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://isasesoria.mx/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1550,58 +1598,62 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Impulsamos personas para que vivan sus mejores oportunidades. Asesoría de inversiones independiente en México, con la fuerza de un grupo de más de 100 oficinas.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>contacto@investsmart.com.mx</t>
+          <t>atencion.al.cliente@finan.mx</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://fmaartini.cl/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1609,53 +1661,57 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+          <t>Flink – Venture Capital</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://apartadomex.com.mx/</t>
+          <t>https://flink.co/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/flink-co/</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>contacto@apartadomex.com.mx</t>
+          <t>info@flink.co</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>Flink app inversión</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1666,12 +1722,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
+          <t>https://www.dineroenimagen.com/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1684,24 +1740,24 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -1712,76 +1768,68 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Plataforma de Beneficios Para Empleados | minu</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.minu.mx/</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="b">
         <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Fideliza y atrae al mejor talento en tu empresa con los beneficios para empleados más valorados. Minu la mejor forma de compensar a tus colaboradores.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/minuservicios/posts/?feedView=all</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>sergio.godinez@minu.mx</t>
-        </is>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>https://godinmx.com/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1789,23 +1837,23 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://misfinanzasdigitales.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1818,36 +1866,40 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>plataforma para invertir en CETES y ETFs México</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ahorro Rinde -</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://ahorrorinde.com.mx/</t>
+          <t>https://fintual.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1860,74 +1912,78 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Jul 27, 2026 · Conoce las mejores plataformas para invertir en México, qué ofrecen, cuánto cuestan y cuál se adapta a tu perfil de inversión.</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
+          <t>Microwd Inversiones - genera impacto social</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://akibaa.com/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.microwd.es/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+          <t>https://www.instagram.com/microwd_inv/</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
+          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+          <t>info@microwd.es</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>Microwd | Microwd</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
@@ -1938,67 +1994,50 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Puntored</t>
+          <t>EMPRENDE PRO MUJER</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://puntored.mx/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Mujeres inversionistas | UBS México</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.ubs.com/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2011,12 +2050,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, mujeres, latam</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -2024,45 +2063,41 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
-        </is>
-      </c>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Rendimientos, ahorro e inversión en México | Ahorro Rinde</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>http://manesseco.com/</t>
+          <t>https://ahorrorinde.com.mx/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia . Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
+          <t>Guías paso a paso sobre rendimientos fintech, Cetes, cuentas de ahorro y fondo de emergencia en México. Aprende a hacer rendir tu dinero hoy.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -2070,14 +2105,10 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
-        </is>
-      </c>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2108,7 +2139,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia . Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2131,12 +2162,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://trocaco.com/</t>
+          <t>http://manesseco.com/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2154,7 +2185,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia . Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
+          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia. Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -2167,7 +2198,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
+          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
         </is>
       </c>
     </row>
@@ -2177,12 +2208,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sanineco | Educación Financiera en Colombia</t>
+          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>http://sanineco.com/</t>
+          <t>https://trocaco.com/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2200,7 +2231,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia . Plataforma líder en análisis de mercados e información económica colombiana.</t>
+          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia. Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -2213,7 +2244,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
+          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
         </is>
       </c>
     </row>
@@ -2223,12 +2254,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bureaco | Educación Financiera en Colombia</t>
+          <t>Sanineco | Educación Financiera en Colombia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>http://bureaco.com/</t>
+          <t>http://sanineco.com/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2246,7 +2277,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
+          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia. Plataforma líder en análisis de mercados e información económica colombiana.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -2259,7 +2290,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
+          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2323,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia . Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras .</t>
+          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia. Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2315,12 +2346,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Bureaco | Educación Financiera en Colombia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>http://larednco.com/</t>
+          <t>http://bureaco.com/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2338,7 +2369,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia . Descubre estrategias de inversión y mejora tu futuro financiero.</t>
+          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2351,7 +2382,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
+          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
         </is>
       </c>
     </row>
@@ -2361,21 +2392,21 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://bitso.com/</t>
+          <t>http://larednco.com/</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2384,26 +2415,22 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
+          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia. Descubre estrategias de inversión y mejora tu futuro financiero.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2411,26 +2438,30 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GBMfondos</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+          <t>https://cashcontrolly.com/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
       <c r="E43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Información sobre fondos de inversión GBM</t>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2438,13 +2469,55 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L43" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Inicio - FIMSE Asesoría Patrimonial Independiente S de RL de CV</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.fimse.com/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, asesoria, regulada, latam</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Conoce FIMSE, Asesores de Inversión Independientes con 30 años de EXPERIENCIA.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>startup mexicana inversión patrimonial personas</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-27
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -500,21 +500,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Perfil | Ultimas noticias de Argentina y el mundo</t>
+          <t>Mujeres y Dinero | educación financiera</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.perfil.com/</t>
+          <t>https://www.mujeres-y-dinero.com/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -522,24 +522,32 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Periodismo Puro: breaking news, análisis y los mejores columnistas cubriendo los temas más importantes de la Argentina y el mundo</t>
+          <t xml:space="preserve">APOYAMOS A MUJERES DE TODAS LAS EDADES PARA QUE APRENDAN A MANEJAR SU DINERO CON CONFIANZA. A veces creemos que los temas vinculados al dinero son “demasiado difíciles” para nosotras.  Desmitifiquemos el tema y tomemos las riendas de nuestra vida financiera. Hay una forma fácil, clara y segura para </t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/perfilcom/</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+          <t>https://www.instagram.com/mujeresydinerouy/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/mujeresydinero/</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>contanos@mujeresydinero.uy</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -600,17 +608,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -618,28 +626,28 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
+          <t>https://www.instagram.com/mujer_financiera/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -650,17 +658,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -668,28 +676,28 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina | Mujer Financiera Argentina</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -735,7 +743,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | app para invertir para principiantes México | app de ahorro e inversión México jóvenes</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -792,21 +800,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bolsa de Chile | IPSA en Tiempo Real | Portal #1 de Inversiones</t>
+          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.bolsadechile.cl/</t>
+          <t>https://www.finamex.com.mx/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -815,15 +823,23 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Cotizaciones IPSA, dólar, UF y fondos mutuos en tiempo real. Educación financiera, calculadoras y comunidad de inversores chilenos. Tu portal financiero de referencia.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -834,21 +850,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.finamex.com.mx/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -857,23 +873,23 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
+          <t>https://www.instagram.com/fintual/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
+          <t>https://www.linkedin.com/company/fintual/</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -884,17 +900,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -902,82 +918,78 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
+          <t>https://www.instagram.com/moradocolombia/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>contacto@morado.app</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>contacto@morado.app</t>
+          <t>hola@eunik.mx</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -988,12 +1000,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1006,24 +1018,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>hola@eunik.mx</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1034,12 +1046,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Inicio - Lakpa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://lakpa.mx/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1052,24 +1064,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>contacto@lakpa.lat</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | plataforma para invertir en CETES y ETFs México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1080,12 +1096,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1098,28 +1114,28 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
-        </is>
-      </c>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1130,46 +1146,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>contacto@asesoresinversion.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma para invertir en CETES y ETFs México</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -1180,17 +1196,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>FG Academia — Educación Financiera e Inversiones para Argentina</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://www.fgacademia.com/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1198,128 +1214,108 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
+          <t>Aprendé a invertir en Argentina con FG Academia. Cursos de finanzas personales, CEDEARs, dólar MEP, cripto y más. Academia online gamificada, simulador de inversiones y mentoría 1:1 con Federico.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="b">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>servicioal.cliente@puntored.co</t>
+          <t>hello@capitellefinance.com</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Inicio - BlockIT Lab</t>
+          <t>Inversiones Chidas | Inversiones y Educación Financiera</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://blockitlab.com/</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>https://inversioneschidas.com/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>El laboratorio donde suceden tus ideas</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/blockitlab/</t>
-        </is>
-      </c>
+          <t>Aprende como invertir con guías paso a paso y material 100% gratis para formarte en temas de inversiones y educación financiera en México.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>proyectos@blockitlab.com</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1330,17 +1326,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Revista Emprendedores | Portada</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://emprendedores.es/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1348,28 +1344,32 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Portada de la Revista Emprendedores.</t>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>fintech inversión mujeres Latinoamérica | fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -1380,46 +1380,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Préstamos personales e inversiones entre personas | yotepresto.com</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.yotepresto.com/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, regulada, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Préstamos personales con las tasas más bajas e inversiones entre personas donde ganas buenos rendimientos. Olvídate de los bancos, ¡conoce yotepresto.com!</t>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/yotepresto-com</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>info@yotepresto.com</t>
-        </is>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -1430,12 +1422,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
+          <t>Mujer Emprende</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://inv.mx/</t>
+          <t>https://www.mujeremprendeglobal.com/</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1448,32 +1440,28 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
+          <t>Escuela de Negocios para Mujeres</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/invierteenseguros/</t>
+          <t>https://www.instagram.com/mujeremprendeglobal</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/invseguros</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>contacto@inv.mx</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/mujer-emprende/</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -1484,42 +1472,50 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Startups Argentina — Directorio y trabajos en el ecosistema startup</t>
+          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.startupsargentina.com/</t>
+          <t>https://inv.mx/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Explorá startups de Argentina, LATAM y Estados Unidos que contratan talento desde Argentina.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/invierteenseguros/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invseguros</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>karen@yafu.app, people@tapi.la</t>
+          <t>contacto@inv.mx</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Mujer Financiera Argentina</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -1580,12 +1576,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Mercadopeso🥇Compara préstamos y tarjetas de crédito</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://www.mercadopeso.mx/</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1598,28 +1594,24 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
+          <t>Mercadopeso México es una empresa de comparación de préstamos y tarjetas de crédito ✅ Mercadopeso es confiable para las mejores opciones y ofertas financieras 🤑</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>atencion.al.cliente@finan.mx</t>
+          <t>info@mercadopeso.mx</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>app para invertir para principiantes México</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -1630,38 +1622,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Inversión Familiar — Educación financiera para familias</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
+          <t>https://inversionfamiliar.es/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="b">
         <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>info@inversionfamiliar.es</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1672,146 +1664,150 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Flink – Venture Capital</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://flink.co/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>En FLINK, nos enorgullecemos de contar con un equipo altamente experimentado en el desarrollo y crecimiento empresarial, el venture capital y la banca de inversión.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/flink-co/</t>
-        </is>
-      </c>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finan.mx/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>info@flink.co</t>
+          <t>atencion.al.cliente@finan.mx</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Flink app inversión</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Franco Martini</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://fmaartini.cl/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
-        </is>
-      </c>
+          <t>Franco Martini</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>https://fundacionana.org/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://marketb2b.mx/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1824,12 +1820,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>mujeres, principiantes, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1837,23 +1833,23 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
+          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://misfinanzasdigitales.com/</t>
+          <t>https://www.bbva.mx/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1866,40 +1862,36 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
-        </is>
-      </c>
+          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1912,108 +1904,100 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/postamx/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Microwd Inversiones - genera impacto social</t>
+          <t>FinTech in Mexico — Inteligencia FinTech México</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.microwd.es/</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>https://www.fintechinmexico.com/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, mujeres, regulada, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Conectamos mujeres emprendedoras en Latinoamérica que solicitan un microcrédito con inversores que buscan rentabilidad económica e impacto social.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/microwd_inv/</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/microwd/?originalSubdomain=co</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>info@microwd.es</t>
-        </is>
-      </c>
+          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Microwd | Microwd</t>
+          <t>Monterrey fintech inversión personas | Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EMPRENDE PRO MUJER</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>https://www.mujeresinvirtiendo.com/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -2024,20 +2008,24 @@
           <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://www.dineroenimagen.com/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2050,54 +2038,54 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Chile</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rendimientos, ahorro e inversión en México | Ahorro Rinde</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://ahorrorinde.com.mx/</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Guías paso a paso sobre rendimientos fintech, Cetes, cuentas de ahorro y fondo de emergencia en México. Aprende a hacer rendir tu dinero hoy.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -2105,28 +2093,28 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>plataforma para invertir en CETES y ETFs México</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>http://www.caraneco.com/</t>
+          <t>https://cashcontrolly.com/</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E36" t="b">
@@ -2134,12 +2122,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2147,45 +2135,41 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://www.caraneco.com/</t>
-        </is>
-      </c>
+          <t>plataforma de inversión para principiantes Perú</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Información sobre negocios financieros en México</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>http://manesseco.com/</t>
+          <t>https://negociosfinancieros.com.mx/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia. Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -2193,165 +2177,169 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
-        </is>
-      </c>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Plataforma de Beneficios Para Empleados | minu</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://trocaco.com/</t>
+          <t>https://www.minu.mx/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia. Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
+          <t>Fideliza y atrae al mejor talento en tu empresa con los beneficios para empleados más valorados. Minu la mejor forma de compensar a tus colaboradores.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/minuservicios/posts/?feedView=all</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>sergio.godinez@minu.mx</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
-        </is>
-      </c>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sanineco | Educación Financiera en Colombia</t>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>http://sanineco.com/</t>
+          <t>https://www.finfit.mx/</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia. Plataforma líder en análisis de mercados e información económica colombiana.</t>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
-        </is>
-      </c>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ramenesco - Educación Financiera en Colombia</t>
+          <t>108 Investments | Gestión Patrimonial e Inversiones</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>http://www.ramenesco.com/</t>
+          <t>https://www.108investments.com.mx/</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia. Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>108 Investments — firma mexicana de gestión patrimonial e inversiones. Tu capital en equilibrio generando valor. Mercados financieros, capital privado y educación financiera.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/108investments?utm_source=qr</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Info@108investments.com</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://www.ramenesco.com/</t>
-        </is>
-      </c>
+          <t>startup mexicana inversión patrimonial personas</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bureaco | Educación Financiera en Colombia</t>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>http://bureaco.com/</t>
+          <t>https://losbancos.mx/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2360,108 +2348,108 @@
         </is>
       </c>
       <c r="E41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
-        </is>
-      </c>
+          <t>Monterrey fintech inversión personas</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>http://larednco.com/</t>
+          <t>https://fintual.mx/</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia. Descubre estrategias de inversión y mejora tu futuro financiero.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
-        </is>
-      </c>
+          <t>Fintual | Fintual</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
+          <t>Pilou, la primera plataforma de ahorro e inversión que busca ...</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
+          <t>https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, digital</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+          <t>Apr 17, 2023 · Andrea de la Garza y Patricia Florencia son las creadoras de Pilou, la primera plataforma de ahorro e inversión creada por mujeres, pensada para mujeres</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -2469,41 +2457,41 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile | plataforma de inversión para principiantes Perú</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Inicio - FIMSE Asesoría Patrimonial Independiente S de RL de CV</t>
+          <t>EMPRENDE PRO MUJER</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://www.fimse.com/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>inversion, asesoria, regulada, latam</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Conoce FIMSE, Asesores de Inversión Independientes con 30 años de EXPERIENCIA.</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H44" t="inlineStr"/>
@@ -2511,13 +2499,728 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>47</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>47</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://akibaa.com/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Inicio - Startup México</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://startupmexico.com/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Mejoramos la vida de las personas a través de la innovación y el  emprendimiento Más información ¿Te gustaría llevar tu Startup o empresa al siguiente nivel? En Startup México contamos con una variedad de CONVOCATORIAS que pueden ayudarte. Consultar convocatorias Nuestros aliados nos respaldan Nuest</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/startup_mexico/?hl=es</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://mx.linkedin.com/company/startupmexico</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>--carmen.mendez@startupmexico.com, --ximena.dealba@startupmexico.com, carmen.mendez@startupmexico.com</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
           <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>http://manesseco.com/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E49" t="b">
+        <v>0</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia. Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>41</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>http://www.caraneco.com/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>0</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://www.caraneco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>41</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://trocaco.com/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>0</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia. Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>41</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sanineco | Educación Financiera en Colombia</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>http://sanineco.com/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E52" t="b">
+        <v>0</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia. Plataforma líder en análisis de mercados e información económica colombiana.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>41</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bureaco | Educación Financiera en Colombia</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>http://bureaco.com/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E53" t="b">
+        <v>0</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>41</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ramenesco - Educación Financiera en Colombia</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>http://www.ramenesco.com/</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E54" t="b">
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia. Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://www.ramenesco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>41</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>http://larednco.com/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E55" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia. Descubre estrategias de inversión y mejora tu futuro financiero.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>41</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://bitso.com/</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>41</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://ecosistemastartup.com/</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="E57" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>hola@ecosistemastartup.com</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Guadalajara fintech inversión ahorro | Guadalajara fintech inversión ahorro</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>41</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Home - GBM</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://about.appgbm.com/</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, digital</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gbmplus_/</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gbm-mx</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>41</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L44"/>
+  <autoFilter ref="A1:L59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-28
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -647,7 +647,7 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
+          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -708,12 +708,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://asesoresinversion.com/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -731,19 +731,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/asesores_inv/</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+          <t>contacto@asesoresinversion.com</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -754,21 +758,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ComparaBancaPerú: Compara Tasas Plazo Fijo, Ahorro y CTS 2026</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://comparabancaperu.com/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -777,35 +781,35 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Compara tasas de 50+ bancos y cajas en Perú. Depósitos a plazo fijo, cuentas de ahorro, CTS, préstamos y tarjetas. Datos SBS actualizados septiembre 2026. 100% gratis.</t>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>luisdrive57@gmail.com</t>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Finamex   Casa De Bolsa - Finamex Casa de Bolsa</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.finamex.com.mx/</t>
+          <t>https://eunik.mx/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -818,49 +822,45 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Somos una firma orgullosamente mexicana, líder como proveedora de servicios de acceso al mercado Mexicano de Valores.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>JavaScript:metConfirmar('https://instagram.com/finamexcb')</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>JavaScript:metConfirmar('https://www.linkedin.com/company/casa-de-bolsa-finamex-ciudad-de-m-xico-mxico')</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>hola@eunik.mx</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://fintual.cl/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -868,49 +868,49 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fintual/</t>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Inicio | Morado</t>
+          <t>FG Academia — Educación Financiera e Inversiones para Argentina</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moradocolombia.com/</t>
+          <t>https://www.fgacademia.com/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -918,32 +918,20 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/moradocolombia/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>contacto@morado.app</t>
-        </is>
-      </c>
+          <t>Aprendé a invertir en Argentina con FG Academia. Cursos de finanzas personales, CEDEARs, dólar MEP, cripto y más. Academia online gamificada, simulador de inversiones y mentoría 1:1 con Federico.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Morado fintech Colombia | Morado fintech Colombia</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -954,42 +942,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Capitelle Finance</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>hola@eunik.mx</t>
+          <t>hello@capitellefinance.com</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1000,163 +988,167 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+          <t>https://www.instagram.com/bolsa24real/</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>info@bolsa24.com</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | fintech mexicana para invertir desde poco dinero</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Inicio - Lakpa</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://lakpa.mx/</t>
+          <t>https://puntored.co/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Construyendo la comunidad de Asesores Financieros Independientes más grande de México Una Nueva forma de gestionar Inversiones Nuestro desarrollo tecnológico rompe paradigmas de la asesoría de inversión; los asesores pueden realizar su labor de forma independiente y todos los clientes pueden optar a</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sherpa-wmc/</t>
+          <t>https://www.linkedin.com/company/puntored/</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>contacto@lakpa.lat</t>
+          <t>servicioal.cliente@puntored.co</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Asesor Financiero Certificado AMIB en México | Asesores Inversión</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://asesoresinversion.com/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Asesoría de inversión personalizada en México con un asesor certificado por la AMIB y registrado en CNBV. Invierte con estrategia y rigor, sin humo. Primera consulta gratis.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/asesores_inv/</t>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>contacto@asesoresinversion.com</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Perfil | Noticias de Argentina y el mundo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://www.perfil.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1164,49 +1156,45 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, principiantes, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Leé las últimas noticias de Argentina y el mundo en Perfil.com. Política, economía, deportes, sociedad y más.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/perfilcom/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FG Academia — Educación Financiera e Inversiones para Argentina</t>
+          <t>Revista Emprendedores | Portada</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.fgacademia.com/</t>
+          <t>https://emprendedores.es/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1214,82 +1202,86 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Aprendé a invertir en Argentina con FG Academia. Cursos de finanzas personales, CEDEARs, dólar MEP, cripto y más. Academia online gamificada, simulador de inversiones y mentoría 1:1 con Federico.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+          <t>Portada de la Revista Emprendedores.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://capitellefinance.com/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
-        </is>
-      </c>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>hello@capitellefinance.com</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Inversiones Chidas | Inversiones y Educación Financiera</t>
+          <t>HOME | PulsoSaludable cuidando tu estilo y forma de vida</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://inversioneschidas.com/</t>
+          <t>https://www.pulsosaludable.com/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1302,20 +1294,28 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Aprende como invertir con guías paso a paso y material 100% gratis para formarte en temas de inversiones y educación financiera en México.</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>PulsoSaludable: Tu fuente de información confiable sobre salud, bienestar, nutrición, ejercicio y prevención en diabetes, obesidad, hipertensión y enfermedades cardiovasculares. Cuidando tu estilo de vida</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/wixstudio</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>info@pulsosaludable.com</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://www.fundssociety.com/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1344,32 +1344,28 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
+          <t>https://www.instagram.com/fundssociety/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica | fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -1380,17 +1376,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
+          <t>Inicio | Préstamos seguros para emprendedoras</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.teiainvest.co/</t>
+          <t>https://www.tappoyo.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1398,145 +1394,137 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, educacion, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tappoyofintech/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mujer Emprende</t>
+          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.mujeremprendeglobal.com/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://mente-mujer.com/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Escuela de Negocios para Mujeres</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/mujeremprendeglobal</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/mujer-emprende/</t>
-        </is>
-      </c>
+          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>INV Seguros | Broker de seguros, retiro e inversión</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://inv.mx/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Broker de seguros, fianzas, retiro e inversión con más de 30 años en México. Comparamos opciones, te explicamos y te acompañamos cuando usas tu seguro.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/invierteenseguros/</t>
-        </is>
-      </c>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/invseguros</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>contacto@inv.mx</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://fundacionana.org/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1544,28 +1532,24 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
+          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/fundacionanaec/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -1576,42 +1560,34 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mercadopeso🥇Compara préstamos y tarjetas de crédito</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.mercadopeso.mx/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="b">
         <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mercadopeso México es una empresa de comparación de préstamos y tarjetas de crédito ✅ Mercadopeso es confiable para las mejores opciones y ofertas financieras 🤑</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>info@mercadopeso.mx</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>app para invertir para principiantes México</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -1622,38 +1598,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inversión Familiar — Educación financiera para familias</t>
+          <t>FinTech in Mexico — Inteligencia FinTech México</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://inversionfamiliar.es/</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>https://www.fintechinmexico.com/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
+          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>info@inversionfamiliar.es</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -1664,12 +1640,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://finan.mx/</t>
+          <t>https://www.kuspit.com/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1682,28 +1658,20 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finan.mx/</t>
-        </is>
-      </c>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>atencion.al.cliente@finan.mx</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>roboadvisor México carteras diversificadas</t>
+          <t>Kuspit | Kuspit</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1714,21 +1682,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Inversiones Chidas | Inversiones y Educación Financiera</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://fmaartini.cl/</t>
+          <t>https://inversioneschidas.com/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1737,7 +1705,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Franco Martini</t>
+          <t>Aprende como invertir con guías paso a paso y material 100% gratis para formarte en temas de inversiones y educación financiera en México.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1745,129 +1713,137 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Chile</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://www.dineroenimagen.com/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>El curso “Camino Financiero de la Mujer Emprendedora” bajo la modalidad virtual, fue diseñada especialmente para mujeres que desean fortalecer su autonomía económica, transformar su relación con el dinero y potenciar su liderazgo personal. A través de herramientas prácticas y conceptos financieros clave, aprenderás a gestionar el dinero de manera estratégica, identificar ...</t>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
+          <t>https://www.instagram.com/dineroenimagen/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://marketb2b.mx/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>mujeres, principiantes, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finxard/</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Te acompañamos en cada paso para lograr lo que te propongas | BBVA México</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.bbva.mx/</t>
+          <t>https://cashcontrolly.com/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Vamos contigo en cada decisión. Inicia con una cuenta y accede a más soluciones financieras, desde ahorro hasta un crédito de auto ¿Avanzamos?</t>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1875,69 +1851,61 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>POSTA</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.posta.com.mx/</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="b">
         <v>1</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/postamx/</t>
-        </is>
-      </c>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>asesor de inversión independiente registrado CNBV</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FinTech in Mexico — Inteligencia FinTech México</t>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.fintechinmexico.com/</t>
+          <t>https://godinmx.com/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1950,12 +1918,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -1963,7 +1931,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas | Guadalajara fintech inversión ahorro</t>
+          <t>app de ahorro e inversión México jóvenes</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
@@ -1974,12 +1942,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mujeres Invirtiendo</t>
+          <t>PAN CDMX</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.mujeresinvirtiendo.com/</t>
+          <t>https://www.pancdmx.org.mx/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1997,22 +1965,26 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>Sitio Oficial del PAN CDMX. Partido Acción Nacional en la Ciudad de México.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pan_cdmx/</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>estudios.pancmx@gmail.com</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
-        </is>
-      </c>
+          <t>educación financiera e inversión para mujeres CDMX</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2020,17 +1992,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>POSTA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://www.posta.com.mx/</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E34" t="b">
@@ -2038,24 +2010,24 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>mujeres, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+          <t>Creamos contenidos innovadores dándole un toque cool y 100 por ciento confiable. Llevamos las noticias más destacadas con presencia en 16 estados de México</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
+          <t>https://www.instagram.com/postamx/</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
@@ -2066,68 +2038,72 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>https://losbancos.mx/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>asesor de inversiones independiente CNBV plataforma digital</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
+          <t>Emprende Pro Mujer</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Perú</t>
-        </is>
-      </c>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="b">
         <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2135,41 +2111,41 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Información sobre negocios financieros en México</t>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://negociosfinancieros.com.mx/</t>
+          <t>https://mifinguia.com/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -2177,23 +2153,23 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
+          <t>plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Plataforma de Beneficios Para Empleados | minu</t>
+          <t>Mujeres inversionistas | UBS México</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.minu.mx/</t>
+          <t>https://www.ubs.com/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2206,140 +2182,124 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, latam</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Fideliza y atrae al mejor talento en tu empresa con los beneficios para empleados más valorados. Minu la mejor forma de compensar a tus colaboradores.</t>
+          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/minuservicios/posts/?feedView=all</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>sergio.godinez@minu.mx</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr"/>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+          <t>FINTECH.TV Terminal: Financial Markets. Built Around You.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://www.finfit.mx/</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://terminal.fintech.tv/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, mujeres, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+          <t>FINTECH.TV delivers 24/7 global financial news and programming, with live coverage from the NYSE, ADX and Cboe, plus studios at Canadian University Dubai.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>contacto@finfit.mx</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>fintech de bienestar financiero para empleados México</t>
+          <t>fintech inversión mujeres Latinoamérica | fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>108 Investments | Gestión Patrimonial e Inversiones</t>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://www.108investments.com.mx/</t>
+          <t>http://caraneco.com/</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>108 Investments — firma mexicana de gestión patrimonial e inversiones. Tu capital en equilibrio generando valor. Mercados financieros, capital privado y educación financiera.</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/108investments?utm_source=qr</t>
-        </is>
-      </c>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Info@108investments.com</t>
-        </is>
-      </c>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>startup mexicana inversión patrimonial personas</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr"/>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
+          <t>Investment Management &amp; Financial Services | BlackRock</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://losbancos.mx/</t>
+          <t>https://www.blackrock.com/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2348,879 +2308,114 @@
         </is>
       </c>
       <c r="E41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
+          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/blackrock</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>plataforma de inversión educación financiera Colombia</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+          <t>GBMfondos</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://fintual.mx/</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="b">
         <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/fintualmx/</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/fintual/</t>
-        </is>
-      </c>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Fintual | Fintual</t>
+          <t>GBM+ inversión</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Pilou, la primera plataforma de ahorro e inversión que busca ...</t>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://heraldodemexico.com.mx/</t>
+          <t>https://www.inversionmasrentable.com/</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, digital</t>
+          <t>inversion, educacion, asesoria</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Apr 17, 2023 · Andrea de la Garza y Patricia Florencia son las creadoras de Pilou, la primera plataforma de ahorro e inversión creada por mujeres, pensada para mujeres</t>
+          <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>contacto@inversionmasrentable.com</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://heraldodemexico.com.mx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>47</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>EMPRENDE PRO MUJER</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="b">
-        <v>0</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>inversion, mujeres, educacion</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>47</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>https://mifinguia.com/</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E45" t="b">
-        <v>1</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>47</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Puntored</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>https://puntored.mx/</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E46" t="b">
-        <v>1</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>inversion, educacion, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Somos la red transaccional -que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/puntoredmx/</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>contacto@gestopago.com, contacto@puntored.mx</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>47</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Akiba | Bienestar financiero para empresas en México</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>https://akibaa.com/</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E47" t="b">
-        <v>1</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/akiba/</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>fintech de bienestar financiero para empleados México</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Inicio - Startup México</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>https://startupmexico.com/</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E48" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>inversion, educacion, asesoria, latam</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Mejoramos la vida de las personas a través de la innovación y el  emprendimiento Más información ¿Te gustaría llevar tu Startup o empresa al siguiente nivel? En Startup México contamos con una variedad de CONVOCATORIAS que pueden ayudarte. Consultar convocatorias Nuestros aliados nos respaldan Nuest</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/startup_mexico/?hl=es</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://mx.linkedin.com/company/startupmexico</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>--carmen.mendez@startupmexico.com, --ximena.dealba@startupmexico.com, carmen.mendez@startupmexico.com</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>startup mexicana inversión patrimonial personas</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>41</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Manesseco - Educación Financiera e Inversiones en Colombia</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>http://manesseco.com/</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E49" t="b">
-        <v>0</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Manesseco - Plataforma líder en educación financiera e información de inversiones en Colombia. Descubre las mejores estrategias de inversión y educación financiera adaptadas al mercado colombiano.</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://manesseco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>41</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>http://www.caraneco.com/</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E50" t="b">
-        <v>0</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://www.caraneco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>41</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Trocaco - Educación Financiera e Inversiones en Colombia</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>https://trocaco.com/</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E51" t="b">
-        <v>0</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Trocaco - Tu plataforma de educación financiera e información de inversiones en Colombia. Aprende sobre finanzas personales, oportunidades de inversión y análisis del mercado colombiano.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: https://trocaco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>41</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Sanineco | Educación Financiera en Colombia</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>http://sanineco.com/</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E52" t="b">
-        <v>0</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Sanineco - Educación financiera y oportunidades de inversión en Colombia. Plataforma líder en análisis de mercados e información económica colombiana.</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://sanineco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>41</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Bureaco | Educación Financiera en Colombia</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>http://bureaco.com/</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E53" t="b">
-        <v>0</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Bureaco - Plataforma colombiana de educación financiera y análisis de inversiones. Aprende a gestionar tu presupuesto personal y descubre el potencial del mercado colombiano.</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://bureaco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>41</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Ramenesco - Educación Financiera en Colombia</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>http://www.ramenesco.com/</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E54" t="b">
-        <v>0</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, educacion, latam</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Ramenesco - Educación financiera y herramientas de inversión para Colombia. Aprende a manejar tu dinero, invierte con confianza y alcanza tus metas financieras.</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://www.ramenesco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>41</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Larednco - Educación Financiera e Inversiones en Colombia</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>http://larednco.com/</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="E55" t="b">
-        <v>0</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Larednco - Tu plataforma de confianza para educación financiera e información sobre inversiones en Colombia. Descubre estrategias de inversión y mejora tu futuro financiero.</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://larednco.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>41</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>https://bitso.com/</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="E56" t="b">
-        <v>1</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>https://instagram.com/bitso</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/bitso</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>fintech mexicana para invertir desde poco dinero</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>41</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>https://ecosistemastartup.com/</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Chile</t>
-        </is>
-      </c>
-      <c r="E57" t="b">
-        <v>0</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>inversion, educacion, latam, digital</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>hola@ecosistemastartup.com</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Guadalajara fintech inversión ahorro | Guadalajara fintech inversión ahorro</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>41</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Home - GBM</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>https://about.appgbm.com/</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, asesoria, digital</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/gbmplus_/</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/gbm-mx</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr">
-        <is>
           <t>GBM+ inversión</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>41</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>GBMfondos</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="b">
-        <v>1</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Información sobre fondos de inversión GBM</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>GBM+ inversión</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L59"/>
+  <autoFilter ref="A1:L43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados de la búsqueda 2026-10-29
</commit_message>
<xml_diff>
--- a/resultados/empresas_como_pilou.xlsx
+++ b/resultados/empresas_como_pilou.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empresas como Pilou" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Empresas como Pilou'!$A$1:$L$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -558,17 +558,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Finantres: Aprende a invertir bien y compara plataformas</t>
+          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://finantres.com/</t>
+          <t>https://www.mujer-financiera.com/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E3" t="b">
@@ -576,28 +576,28 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aprende a invertir bien y compara las mejores plataformas con análisis reales, guías paso a paso y sin publicidad engañosa.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mujer_financiera/</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/finantres/</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>contacto@finantres.com</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup | Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -608,17 +608,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mujer Financiera | Cursos de finanzas e inversiones desde cero</t>
+          <t>Visionarias Business - Visionarias Business</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.mujer-financiera.com/</t>
+          <t>https://visionarias.business/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -626,78 +626,74 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aprendé a ordenar tus finanzas, ahorrar e invertir con cursos simples y en español. Más de 800.000 alumnas aprendieron con MF desde 2018. Armá tu presupuesto, hacé tu primera inversión y armá una estrategia para invertir en tu retiro. Acompañada por asesores y expertos en el mercado.</t>
+          <t>«La revolución de las mujeres en Fintech y Femtech está reconfigurando el sistema financiero con innovación, liderazgo y propósito. Desde el crecimiento de fundadoras y ejecutivas en todo el mundo, hasta el desarrollo de tecnologías con enfoque de género, el impacto femenino se extiende a la inclusión financiera, la inversión estratégica y la creación de redes de apoyo. Este ...</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mujer_financiera/</t>
+          <t>https://www.instagram.com/visionarias.business/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mujer-financiera/</t>
+          <t>https://www.linkedin.com/company/visionarias</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup | educación financiera para mujeres invertir startup</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Visionarias Business - Visionarias Business</t>
+          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://visionarias.business/</t>
+          <t>https://finantres.mx/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>El crecimiento del ecosistema Fintech y Femtech no sería posible sin el impulso de fondos de inversión con enfoque de género y redes de apoyo que promueven el liderazgo femenino; estas plataformas fortalecen el ecosistema emprendedor femenino, generando condiciones para una participación más equitativa y estratégica.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/visionarias.business/</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/visionarias</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>app para invertir para principiantes México | app para invertir para principiantes México | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -747,7 +743,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>asesor de inversiones independiente CNBV plataforma digital | roboadvisor México carteras diversificadas | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -758,21 +754,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Finantres México: Te ayuda a encontrar tu plataforma de inversión</t>
+          <t>Bolsa de Chile | IPSA en Tiempo Real | Portal #1 de Inversiones</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://finantres.mx/</t>
+          <t>https://www.bolsadechile.cl/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -781,86 +777,82 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Finantres México te ayuda a encontrar la plataforma de inversión perfecta para ti, de manera sencilla y sin rodeos. Hemos llegado para revolucionar la industria, pero, sobre todo, para apoyarte.</t>
+          <t>Cotizaciones IPSA, dólar, UF y fondos mutuos en tiempo real. Educación financiera, calculadoras y comunidad de inversores chilenos. Tu portal financiero de referencia.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>aleborjafu@gmail.com, contacto@finantres.com</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>plataforma de inversión para principiantes Chile</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
+          <t>Perfil | Noticias de Argentina y el mundo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://eunik.mx/</t>
+          <t>https://www.perfil.com/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, ahorro, mujeres, principiantes, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>Leé las últimas noticias de Argentina y el mundo en Perfil.com. Política, economía, deportes, sociedad y más.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/perfilcom/</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>hola@eunik.mx</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México | plataforma de inversión para mujeres México</t>
+          <t>fintech inversión Argentina principiantes | fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Invierte en tu Futuro | el fondo</t>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.el-fondo.com/</t>
+          <t>https://fintual.cl/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="E9" t="b">
@@ -868,49 +860,49 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
+          <t>Fintual es la app líder en inversiones reguladas en la región: +200 mil personas invierten fácil y sin mínimos en fondos, APV, acciones y ETFs.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/elfondo.inversiones/</t>
+          <t>https://www.instagram.com/fintual/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+          <t>https://www.linkedin.com/company/fintual/</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>Fintual | Fintual</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FG Academia — Educación Financiera e Inversiones para Argentina</t>
+          <t>Inicio | Morado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.fgacademia.com/</t>
+          <t>https://www.moradocolombia.com/</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" t="b">
@@ -918,20 +910,32 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Aprendé a invertir en Argentina con FG Academia. Cursos de finanzas personales, CEDEARs, dólar MEP, cripto y más. Academia online gamificada, simulador de inversiones y mentoría 1:1 con Federico.</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+          <t>Morado ofrece soluciones de crédito flexibles y estratégicas para impulsar negocios, además de productos de belleza y financiamiento para emprendedoras en América Latina.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/moradocolombia/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://co.linkedin.com/company/moradoweb&amp;ved=2ahUKEwjvoc_VibqLAxUpRTABHT2iALwQFnoECAkQAQ&amp;usg=AOvVaw3dE0oCYMWsMrcbtNFfbn9g</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>contacto@morado.app</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>Morado fintech Colombia | Morado fintech Colombia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -942,42 +946,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
+          <t>Asesoría Financiera para Mujeres en México | Eunik</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://capitellefinance.com/</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>https://eunik.mx/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
+          <t>inversion, ahorro, mujeres, educacion, asesoria, latam</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Capitelle Finance</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
-        </is>
-      </c>
+          <t>En Eunik, transformamos la cultura financiera en México a través de asesoría especializada en inversiones, enfocándonos en empoderar a las mujeres para que tomen decisiones financieras informadas.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>hello@capitellefinance.com</t>
+          <t>hola@eunik.mx</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>educación financiera para mujeres invertir startup</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -988,12 +992,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
+          <t>Club privado de inversión para mujeres | Inversoras Club</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.bolsa24.net/</t>
+          <t>https://inversoras.club/</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1006,103 +1010,99 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
+          <t>inversion, mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+          <t>Club privado de inversión para mujeres. Más de 2.600 socias comparten experiencias y contactos en un entorno exclusivo.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/bolsa24real/</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>https://www.instagram.com/club_inversoras/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/inversoras-club/</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>info@bolsa24.com</t>
+          <t>info@inversoras.club</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Kuspit</t>
+          <t>plataforma de inversión para mujeres México</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
+          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://puntored.co/</t>
+          <t>https://alquimistadeldinero.com/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/puntoredcolombia/</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/puntored/</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>servicioal.cliente@puntored.co</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/alquimista_del_dinero/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>app para invertir para principiantes México | plataforma de inversión para principiantes Perú | fintech mexicana para invertir desde poco dinero</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alquimista del Dinero — Finanzas personales claras para Latinoamérica</t>
+          <t>Invierte en tu Futuro | el fondo</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://alquimistadeldinero.com/</t>
+          <t>https://www.el-fondo.com/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Perú</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1110,20 +1110,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, asesoria, latam</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Finanzas personales claras y sin humo para Latinoamérica: cómo ahorrar, invertir desde cero, salir de deudas y generar ingresos extra.</t>
+          <t>La plataforma líder de datos y educación financiera para Latinoamérica: El Fondo reúne acciones, ETF, cripto y divisas con datos de nivel institucional, explicados con claridad. Explora, compara y aprende a invertir con confianza.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/alquimista_del_dinero/</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>https://www.instagram.com/elfondo.inversiones/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/el-fondo-com-1/</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
@@ -1134,21 +1138,21 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Perfil | Noticias de Argentina y el mundo</t>
+          <t>Inversiones24: Tu Portal de Confianza para Invertir desde Latinoamérica</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.perfil.com/</t>
+          <t>https://www.inversiones24.com/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1156,45 +1160,45 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>inversion, mujeres, principiantes, empresas_b2b, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Leé las últimas noticias de Argentina y el mundo en Perfil.com. Política, economía, deportes, sociedad y más.</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/perfilcom/</t>
-        </is>
-      </c>
+          <t>Descubre en Inversiones24 las mejores plataformas de inversión, brokers regulados, cursos y guías para aprender a invertir en bolsa, acciones, ETF y criptomonedas.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>info@colonna-global-media.com</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>fintech inversión Argentina principiantes</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Revista Emprendedores | Portada</t>
+          <t>FG Academia — Educación Financiera e Inversiones para Argentina</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://emprendedores.es/</t>
+          <t>https://www.fgacademia.com/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1202,191 +1206,191 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, digital</t>
+          <t>inversion, ahorro, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Portada de la Revista Emprendedores.</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
-        </is>
-      </c>
+          <t>Aprendé a invertir en Argentina con FG Academia. Cursos de finanzas personales, CEDEARs, dólar MEP, cripto y más. Academia online gamificada, simulador de inversiones y mentoría 1:1 con Federico.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
+          <t>Capitelle Finance</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://becasbenitojuarezmx.com/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
+          <t>https://capitellefinance.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, principiantes, educacion, empresas_b2b</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
+          <t>Capitelle Finance</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/capitellefinance?igsh=MWdpYnM5eGdnZnVpaQ==</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>hello@capitellefinance.com</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HOME | PulsoSaludable cuidando tu estilo y forma de vida</t>
+          <t>Revista Emprendedores | Portada</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.pulsosaludable.com/</t>
+          <t>https://emprendedores.es/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, asesoria, latam</t>
+          <t>inversion, mujeres, educacion, asesoria, empresas_b2b, digital</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>PulsoSaludable: Tu fuente de información confiable sobre salud, bienestar, nutrición, ejercicio y prevención en diabetes, obesidad, hipertensión y enfermedades cardiovasculares. Cuidando tu estilo de vida</t>
+          <t>Portada de la Revista Emprendedores.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/wixstudio</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>info@pulsosaludable.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/revista_emprendedores/?hl=es</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/company/revista-emprendedores-spain</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>fintech ahorro e inversión mujeres emprendedoras</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Asesores Financieros en México | Retiro, Inversión y Seguros | EB Consulting</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.fundssociety.com/</t>
+          <t>https://www.ebconsultingmx.com/</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+          <t>Asesoría Financiera personalizada en México. Diseñamos estrategias de inversión y retiro para construir y proteger tu patrimonio. Agenda tu asesoría sin costo.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundssociety/</t>
+          <t>https://www.instagram.com/eltiofinanciero/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/funds-society/</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
+          <t>https://www.linkedin.com/company/ebconsultingmx/?viewAsMember=true</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>solicitudes@ebconsultingmx.com</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Inicio | Préstamos seguros para emprendedoras</t>
+          <t>Startups Argentina — Directorio y trabajos en el ecosistema startup</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.tappoyo.com/</t>
+          <t>https://www.startupsargentina.com/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1394,86 +1398,94 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tappoyo impulsa la inclusión financiera de mujeres emprendedoras mediante préstamos seguros, tecnología, comunidad e inversión de impacto en Perú.</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/tappoyofintech/</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/tappoyo/?viewAsMember=true</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
+          <t>Explorá startups de Argentina, LATAM y Estados Unidos que contratan talento desde Argentina.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>karen@yafu.app, people@tapi.la</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Tappoyo Perú | Tappoyo Perú | Tappoyo Perú</t>
+          <t>Mujer Financiera Argentina</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3 plataformas de ahorro e inversión que hacen crecer tu dinero</t>
+          <t>Puntored:Plataforma de pagos impulsa la inclusión financiera</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://mente-mujer.com/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>https://puntored.co/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E21" t="b">
         <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, principiantes, digital</t>
+          <t>inversion, mujeres, educacion, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hoy existen más oportunidades para que las mujeres gestionen su dinero con autonomía y visión de futuro. Estas plataformas de ahorro e inversión permiten empezar desde cero y construir un camino financiero con poder personal y sostenido. No necesitas grandes sumas: incluso con 100 pesos al mes, puedes activar el interés compuesto a tu favor.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+          <t>Puntored conecta a millones de personas y negocios con servicios financieros digitales, pagos masivos y corresponsalía bancaria en LATAM.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredcolombia/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored/</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>servicioal.cliente@puntored.co</t>
+        </is>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>403 Client Error: Forbidden for url: https://mente-mujer.com/</t>
-        </is>
-      </c>
+          <t>fintech inversión mujeres Latinoamérica</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
+          <t>Teia Invest | Educación financiera e inversiones para mujeres en Colombia y LATAM</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://colcapital.org/</t>
+          <t>https://www.teiainvest.co/</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1486,45 +1498,41 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
+          <t>Teia Invest es la comunidad de educación financiera e inversiones para mujeres en Colombia y LATAM. Cursos, herramientas y comunidad. +60K mujeres en +60 países.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/colcapital</t>
-        </is>
-      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>educación financiera para mujeres invertir startup</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fundación Ana – Cuando una ecuatoriANA progresa, impulsa el crecimiento de su familia, su comunidad y su país.</t>
+          <t>iProfesional | Últimas noticias para profesionales y empresas</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://fundacionana.org/</t>
+          <t>https://www.iprofesional.com/</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1532,21 +1540,29 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam, digital</t>
+          <t>inversion, mujeres, principiantes, educacion, latam</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>¿Estás lista para llevar tu emprendimiento al siguiente nivel y tomar el control total de tus finanzas? Este curso está pensado para mujeres que quieren aprender a cuidar su dinero, invertirlo bien y hacer su negocio más fuerte, fue diseñado por Cooperativa Andalucía.</t>
+          <t>Últimas noticias sobre economía, política, finanzas, impuestos, Inteligencia Artificial, criptomonedas, inversiones y dólar</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fundacionanaec/</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+          <t>https://www.instagram.com/iProfesional/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/iprofesional-com/</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>asanguinetti@iprofesional.com, cdergarabedian@iprofesional.com, claudiozlotnik@gmail.com</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>educación financiera para mujeres invertir startup</t>
@@ -1556,30 +1572,34 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Home | Minerva Educación Financiera</t>
+          <t>BECAS BENITO JUÁREZ 2025: Requisitos, REGISTRO y FECHAS de pago 📅</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.minervaeducacionfinanciera.mx/</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>https://becasbenitojuarezmx.com/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E24" t="b">
         <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>inversion, ahorro, mujeres, educacion, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
+          <t>Consulta todo sobre las BECAS BENITO JUÁREZ 2025. Revisa REQUISITOS, haz tu REGISTRO y conoce las FECHAS de pago oficiales. ¡Haz clic y entérate ahora!</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1594,16 +1614,16 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FinTech in Mexico — Inteligencia FinTech México</t>
+          <t>INV Seguros: compara y contrata seguros, retiro e inversión</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.fintechinmexico.com/</t>
+          <t>https://inv.mx/</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1616,62 +1636,82 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+          <t>Más de 30 años comparando aseguradoras para ti. Cotiza, compara y contrata con un asesor que te acompaña el día que usas tu seguro. Regulados por la CNSF.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/invierteenseguros/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invseguros</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>contacto@inv.mx</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kuspit | Inversión para principiantes y expertos</t>
+          <t>Bolsa24: Análisis y Comparativas de brokers para invertir con confianza</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.kuspit.com/</t>
+          <t>https://www.bolsa24.net/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>España</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>Bolsa24 es tu portal de confianza para elegir los mejores brokers: análisis profesionales, rankings independientes y metodología transparente.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bolsa24real/</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>info@bolsa24.com</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Kuspit | Kuspit</t>
+          <t>Kuspit</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -1682,54 +1722,58 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Inversiones Chidas | Inversiones y Educación Financiera</t>
+          <t>ColCapital | Asociación Colombiana de Capital Privado</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://inversioneschidas.com/</t>
+          <t>https://colcapital.org/</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inversion, ahorro, principiantes, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Aprende como invertir con guías paso a paso y material 100% gratis para formarte en temas de inversiones y educación financiera en México.</t>
+          <t>ColCapital es la Asociación Colombiana de Capital Privado. Actualmente cuenta con 166 miembros, de los cuales 83 son gestores profesionales y otros vehículos de inversión y 83 son proveedores de servicios de la industria.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/colcapital</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DineroenImagen</t>
+          <t>Préstamos Personales en Línea Finan.mx - Créditos Confiables</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.dineroenimagen.com/</t>
+          <t>https://finan.mx/</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1742,95 +1786,91 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>mujeres, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+          <t>Finan te ofrece préstamos en línea desde el 0% de intereses, desde tu casa y sin burocracia. Consigue ya tu préstamo con Finan.mx</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/dineroenimagen/</t>
+          <t>https://www.instagram.com/finan.mx/</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>atencion.al.cliente@finan.mx</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
+          <t>Inversión Familiar — Educación financiera para familias</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://finxard.com/</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://inversionfamiliar.es/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="b">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, principiantes, educacion, asesoria, regulada</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/finxard/</t>
-        </is>
-      </c>
+          <t>Aprende a invertir con cabeza: fondos indexados, ETFs, acciones y fiscalidad explicados para familias. Calculadoras, glosario, sección infantil y asesor financiero gratuito.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>contacto@finxard.com, johndoe@gmail.com</t>
+          <t>info@inversionfamiliar.es</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
+          <t>roboadvisor México carteras diversificadas</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CashControlly · End the month with money, not red numbers</t>
+          <t>Últimas noticias de Argentina y el mundo - LA NACION</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://cashcontrolly.com/</t>
+          <t>https://www.lanacion.com.ar/</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Perú</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="E30" t="b">
@@ -1838,36 +1878,44 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>inversion, principiantes, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>LA NACION ofrece las últimas noticias, fotos y videos de la Argentina y el mundo. Política, economía, deportes y toda la información en tiempo real.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lanacioncom/</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>LNJuegos@lanacion.com.ar, jalvarez@lanacion.com.ar, jrizzo@lanacion.com.ar</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>plataforma de inversión para principiantes Perú</t>
+          <t>fintech inversión Argentina principiantes</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
+          <t>Home | Minerva Educación Financiera</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://softcredito.com.mx/</t>
+          <t>https://www.minervaeducacionfinanciera.mx/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1876,12 +1924,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, regulada, digital</t>
+          <t>inversion, ahorro, mujeres, educacion, digital</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
+          <t>Proyecto Minerva. Educación financiera con perspectiva de género.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1889,23 +1937,23 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>asesor de inversión independiente registrado CNBV</t>
+          <t>educación financiera e inversión para mujeres CDMX</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+          <t>Abogados en CDMX — Despacho Jurídico Especializado en Derecho Familiar, Civil, Penal y Corporativo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://godinmx.com/</t>
+          <t>https://abogadosencdmx.com/</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1918,36 +1966,48 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, regulada, latam</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+          <t>Despacho jurídico en Roma Norte, CDMX. Especialistas en derecho familiar, penal, civil, corporativo, migratorio, inmobiliario y laboral. Consulta gratuita.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://instagram.com/abogadosencdmx</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/company/abogadosencdmx</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>contacto@abogadosencdmx.com</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>app de ahorro e inversión México jóvenes</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAN CDMX</t>
+          <t>Microsip – El ERP hecho para tu empresa ¡Maximiza el potencial!</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.pancdmx.org.mx/</t>
+          <t>https://www.microsip.com/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1960,35 +2020,35 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion, latam</t>
+          <t>inversion, ahorro, educacion, asesoria, empresas_b2b, latam</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sitio Oficial del PAN CDMX. Partido Acción Nacional en la Ciudad de México.</t>
+          <t>Toma el control, elige las mejores decisiones y alcanza todas tus metas con un ERP hecho para tu empresa. Nómina, contabilidad, inventarios,</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/pan_cdmx/</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>estudios.pancmx@gmail.com</t>
-        </is>
-      </c>
+          <t>https://www.instagram.com/microsip/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microsip/?originalSubdomain=mx</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>educación financiera e inversión para mujeres CDMX</t>
+          <t>startup mexicana inversión patrimonial personas</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2002,7 +2062,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E34" t="b">
@@ -2010,7 +2070,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>mujeres, principiantes, educacion, latam, digital</t>
+          <t>inversion, mujeres, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2034,21 +2094,21 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
+          <t>FinTech in Mexico — Inteligencia FinTech México</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://losbancos.mx/</t>
+          <t>https://www.fintechinmexico.com/</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E35" t="b">
@@ -2056,120 +2116,136 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>inversion, educacion, asesoria, latam, digital</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
-        </is>
-      </c>
+          <t>Inteligencia FinTech México: noticias, fusiones y adquisiciones, directorio de empresas, comparador independiente y reportes del ecosistema fintech mexicano.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Monterrey fintech inversión personas</t>
+          <t>Monterrey fintech inversión personas | Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer</t>
+          <t>Funds Society - Punto de encuentro para la industria de Asset y Wealth Management</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://emprendepromujer.org/</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>https://www.fundssociety.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
       <c r="E36" t="b">
         <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>inversion, mujeres, educacion</t>
+          <t>inversion, educacion, asesoria, empresas_b2b, latam, digital</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>Punto de encuentro para la industria de Asset y Wealth Management</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fundssociety/</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/funds-society/</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>plataforma de inversión para mujeres México</t>
+          <t>Monterrey fintech inversión personas</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+          <t>Finanzas Transparentes | Finsus</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://mifinguia.com/</t>
+          <t>https://finsus.mx/</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>inversion, ahorro, educacion, latam, digital</t>
+          <t>inversion, ahorro, asesoria, empresas_b2b, regulada, latam, digital</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>SOFIPO líder en México, especializada en ahorro e inversión con rendimientos competitivos y total seguridad. Abre tu cuenta en minutos y haz crecer tu dinero de forma simple, confiable y sin complicaciones.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finsusapp</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>info@finsus.mx</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Perú</t>
+          <t>Guadalajara fintech inversión ahorro</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mujeres inversionistas | UBS México</t>
+          <t>Mujeres Invirtiendo</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.ubs.com/</t>
+          <t>https://www.mujeresinvirtiendo.com/</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2182,12 +2258,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>inversion, mujeres, latam</t>
+          <t>inversion, mujeres, educacion, latam</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Comprendemos las necesidades de inversión de las mujeres y les proporcionamos las herramientas para tomar el control de su futuro financiero.</t>
+          <t>Somos una comunidad de +300 mujeres trabajando activamente en la industria de Inversiones en México, a través de +90 Instituciones en Private Equity, Venture Capital, Aceleradoras e Incubadoras, Family Offices, Inversionistas Institucionales e Inversionistas Ángeles.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -2200,78 +2276,82 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>403 Client Error: Forbidden for url: https://www.ubs.com/</t>
+          <t>HTTPSConnectionPool(host='www.mujeresinvirtiendo.com', port=443): Max retries exceeded with url: / (Caused by NewConnect</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FINTECH.TV Terminal: Financial Markets. Built Around You.</t>
+          <t>DineroenImagen</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://terminal.fintech.tv/</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>https://www.dineroenimagen.com/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
       <c r="E39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>inversion, mujeres, digital</t>
+          <t>mujeres, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>FINTECH.TV delivers 24/7 global financial news and programming, with live coverage from the NYSE, ADX and Cboe, plus studios at Canadian University Dubai.</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr"/>
+          <t>Dinero en Imagen te da noticias sobre economía, finanzas personales, negocios, tecnología, compra de autos, divisas, precio del dólar, análisis financieros y de mercado</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dineroenimagen/</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>fintech inversión mujeres Latinoamérica | fintech ahorro e inversión mujeres emprendedoras</t>
+          <t>fintech inversión mujeres Latinoamérica</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+          <t>Software de Crédito - Administra tu cartera - Software para Sofom</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>http://caraneco.com/</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+          <t>https://softcredito.com.mx/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, regulada, digital</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+          <t>Software de Crédito para entidades Financieras.Tenemos la solución de la Administración de cartera, administración de riesgos y PLD. ¡DEMO GRATIS!</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2279,27 +2359,23 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>plataforma de inversión educación financiera Colombia</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
-        </is>
-      </c>
+          <t>asesor de inversiones independiente CNBV plataforma digital | asesor de inversión independiente registrado CNBV</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Investment Management &amp; Financial Services | BlackRock</t>
+          <t>Finxard | Plataforma de Inversión y Análisis Bursátil en Colombia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://www.blackrock.com/</t>
+          <t>https://finxard.com/</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2312,21 +2388,25 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>inversion, educacion, latam, digital</t>
+          <t>inversion, educacion, asesoria, latam, digital</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/blackrock</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
+          <t>Formación bursátil con método académico. Datos, herramientas y comunidad. Más de 3.500 estudiantes ya usan la app.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/finxard/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>contacto@finxard.com, johndoe@gmail.com</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>plataforma de inversión educación financiera Colombia</t>
@@ -2336,30 +2416,34 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GBMfondos</t>
+          <t>CashControlly · End the month with money, not red numbers</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://gbmfondos.com.mx/</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>https://cashcontrolly.com/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Perú</t>
+        </is>
+      </c>
       <c r="E42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+          <t>inversion, principiantes, educacion, latam, digital</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Información sobre fondos de inversión GBM</t>
+          <t>Personal finance app. Budgets, savings goals, scheduled expenses. 14-day free trial, no card required.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -2367,55 +2451,1306 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>GBM+ inversión</t>
+          <t>plataforma de inversión para principiantes Perú</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+          <t>EbankingNews by Digital Bank LATAM</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://www.inversionmasrentable.com/</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+          <t>http://ebankingnews.com/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
       <c r="E43" t="b">
         <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Lo último en banca, tecnología y negocios en tiempo real. Descubre startups Fintech y análisis de los líderes que marcan el futuro del eBanking.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/grupodigitalbank/</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/digital-bank-latam/</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>fintech inversión Argentina principiantes</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>53</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Información sobre negocios financieros en México</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://negociosfinancieros.com.mx/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Descubre información sobre negocios financieros en México, con guías y análisis para optimizar tus decisiones y recursos.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>53</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ApartadoMex — Finanzas, IA, CETES y SAT para México 2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://apartadomex.com.mx/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Portal de inteligencia financiera para México: análisis gubernamental, inversión y herramientas de IA para decisiones más inteligentes con tu dinero.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>contacto@apartadomex.com.mx</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>53</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Tiendanube | Creá gratis tu tienda online</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.tiendanube.com/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>0</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>El mejor diseño para tu marca, 100+ aplicaciones para potenciar tu tienda y soporte humano cuando necesites. Vendé con la plataforma de e-commerce más elegida de Argentina.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tiendanube.arg/</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tiendanube/</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>53</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>GodinMX — Todo para el godín mexicano | GodinMX</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://godinmx.com/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Calculadoras de derechos laborales, guías LFT, comunidad de trabajadores, fondas, juegos y lo que necesitas saber sin que tu jefe lo sepa.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>app de ahorro e inversión México jóvenes</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>53</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PAN CDMX</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.pancdmx.org.mx/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, educacion, latam</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Sitio Oficial del PAN CDMX. Partido Acción Nacional en la Ciudad de México.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pan_cdmx/</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>estudios.pancmx@gmail.com</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>educación financiera e inversión para mujeres CDMX</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>53</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Mejores tasas de CETES, SOFIPOs y bancos | Mis Finanzas Digitales</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://misfinanzasdigitales.com/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Compara las mejores tasas de CETES, SOFIPOs y bancos en México. Encuentra dónde gana más tu dinero sin riesgo. Actualizado cada semana.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ricardofinanzasdigitales/</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>53</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Guías de Viaje</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://guiasdeviaje.mx/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Guías completas de México y el mundo — destinos, pueblos mágicos, playas y rutas gastronómicas con consejos reales para viajeros.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>53</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Finfit — Cajas y fondos de ahorro laborales | Bienestar financiero</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.finfit.mx/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Finfit: ecosistema digital de bienestar financiero laboral. Caja de ahorro, fondo de ahorro, pago de servicios y seguros para tus colaboradores.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>contacto@finfit.mx</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>53</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>108 Investments | Gestión Patrimonial e Inversiones</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.108investments.com.mx/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>108 Investments — firma mexicana de gestión patrimonial e inversiones. Tu capital en equilibrio generando valor. Mercados financieros, capital privado y educación financiera.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/108investments?utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Info@108investments.com</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>startup mexicana inversión patrimonial personas</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>53</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>losbancos.mx - Noticias del sistema bancario mexicano.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://losbancos.mx/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>inversion, educacion, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Noticias del sistema bancario mexicano. Bancos de México. Noticias del sistema bancario mexicano. Calificación de préstamos, hipotecarios.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lettveicom/?igsh=YXZhdTIxZmpibjVz</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Monterrey fintech inversión personas</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Invertir es así de simple, tus inversiones reguladas - Fintual</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://fintual.mx/</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, regulada, latam, digital</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Organiza tus ahorros invirtiendo en alternativas simples y reguladas por la CNBV, con comisiones bajas. Sin papeleos ni letra chica.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fintualmx/</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fintual/</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Fintual | Fintual</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Kuspit | Inversión para principiantes y expertos</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://kuspit.com/</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, asesoria, latam, digital</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Invierte desde México en Acciones de todo el mundo, CETES, ETF's y más con la comisión más baja del mercado.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Kuspit | Kuspit</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EMPRENDE PRO MUJER</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://emprendepromujer.org/</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="b">
+        <v>0</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>inversion, mujeres, educacion</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Emprende Pro Mujer es parte de Pro Mujer una empresa social que durante más de 33 años ha apoyado a que las mujeres alcancen su máximo potencial, a través de la inclusión financiera y digital, servicios de salud y educación. Emprende es una comunidad digital donde las mujeres pueden fortalecer sus habilidades personales y para el emprendimiento y así alcanzar su prosperidad económica ...</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para mujeres México</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>47</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>MiFinGuía — Bancos, seguros y herramientas en español</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://mifinguia.com/</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Compara cuentas bancarias y seguros con fuentes oficiales. Guías para Perú, México y Colombia, directorio financiero y calculadoras en español.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas | plataforma de inversión educación financiera Colombia | plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>47</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Rendimientos, ahorro e inversión en México | Ahorro Rinde</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://ahorrorinde.com.mx/</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Guías paso a paso sobre rendimientos fintech, Cetes, cuentas de ahorro y fondo de emergencia en México. Aprende a hacer rendir tu dinero hoy.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>plataforma para invertir en CETES y ETFs México</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>47</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Marketb2b - es un marketplace B2B de productos industriales y de consumo</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://marketb2b.mx/</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>mujeres, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Marketplace B2B |  Publica tus productos | Sin comisiones | Generamos tráfico orgánico hacia tus productos | Incremeta tus ventas.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México | fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>47</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Puntored</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://puntored.mx/</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E60" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>inversion, educacion, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Somos la red transaccional +que conecta lo físico con lo digital, acercando servicios financieros a más personas, comercios y empresas en América Latina.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/puntoredmx/</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/puntored-gestopago-mexico/</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>contacto@gestopago.com, contacto@puntored.mx</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Akiba | Bienestar financiero para empresas en México</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://akibaa.com/</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E61" t="b">
+        <v>1</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ahorro, educacion, asesoria, empresas_b2b, latam, digital</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Plataforma de bienestar financiero para empresas: caja y fondo de ahorro, sueldo anticipado y educación financiera en una sola app.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/akibamexico?igsh=MW82bnpmM2tqcXZrdw==</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/akiba/</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>info@akibaa.com, minombre@mail.com, ventas@akibaa.com</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>fintech de bienestar financiero para empleados México</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>41</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Inversión Más Rentable | Trading Algorítmico e IA Financiera | Inversión Más Rentable</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.inversionmasrentable.com/</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t>inversion, educacion, asesoria</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>Expertos en trading algorítmico, inteligencia artificial para inversiones y consultoría financiera. Maximiza tus rendimientos con tecnología de punta.</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
         <is>
           <t>contacto@inversionmasrentable.com</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>roboadvisor México carteras diversificadas</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>41</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Caraneco - Educación Financiera e Inversión en Colombia</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>http://caraneco.com/</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E63" t="b">
+        <v>0</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Caraneco - Plataforma de educación financiera e inversión en Colombia. Aprende sobre finanzas personales, mercados y construye tu patrimonio.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>404 Client Error: Not Found for url: http://caraneco.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>41</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Investment Management &amp; Financial Services | BlackRock</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.blackrock.com/</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="E64" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>BlackRock is one of the world’s preeminent asset management firms and a premier provider of investment management. Find out more information here.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/blackrock</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>plataforma de inversión educación financiera Colombia</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>41</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Wise: The international account | Money without borders | Wise United States</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://wise.com/</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="E65" t="b">
+        <v>0</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>150+ countries, 40 currencies, one account. Save when you send, spend and manage your money internationally.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/wiseaccount</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/company/wiseaccount</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>ouvidoria@wise.com, u003eouvidoria@wise.com</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>plataforma de inversión para principiantes Chile</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>41</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Crypto and Stock Investing App | Buy, Sell &amp; Earn | Bitso</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://bitso.com/</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E66" t="b">
+        <v>1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Invest in crypto, bitcoin, ethereum, and global stocks. Earn yields, send, and receive money securely with Bitso. Join millions, growing their money with one powerful app.</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://instagram.com/bitso</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bitso</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>41</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Chatterize - Get the best financial products on the market</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://chatterize.com/</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>inversion, principiantes, latam, digital</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Get the best financial products on the market</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>fintech mexicana para invertir desde poco dinero</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>41</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Startups, tecnología e IA en español | El Ecosistema Startup</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://ecosistemastartup.com/</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="E68" t="b">
+        <v>1</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>inversion, educacion, latam, digital</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>El medio del ecosistema emprendedor hispanohablante: startups, tecnología, inteligencia artificial y financiamiento, cada día.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/elecosistemastartup/</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>hola@ecosistemastartup.com</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>startup mexicana inversión patrimonial personas | Guadalajara fintech inversión ahorro | Guadalajara fintech inversión ahorro</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>41</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Home - GBM</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://about.appgbm.com/</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="b">
+        <v>0</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, asesoria, digital</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar Descarga la nueva app de GBM y (r)evoluciona tus inversiones.  Conoce más Descargar Descargar La nueva app de GBM tiene un diseño innovador para mejorar tu experiencia al momento de explorar e invertir en l</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gbmplus_/</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/gbm-mx</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
         <is>
           <t>GBM+ inversión</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>41</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>GBMfondos</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://gbmfondos.com.mx/</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="b">
+        <v>1</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>inversion, ahorro, empresas_b2b, regulada, digital</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Información sobre fondos de inversión GBM</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>GBM+ inversión</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:L70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>